<commit_message>
062325 - updated skins docs
</commit_message>
<xml_diff>
--- a/public/results/2025/2025 Weekly Stats - Week 7.xlsx
+++ b/public/results/2025/2025 Weekly Stats - Week 7.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="615" documentId="13_ncr:1_{D28DBAEF-3652-6147-89B5-C7FAD277D708}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BD5B83FF-B0A2-4637-AA82-E55A2226A389}"/>
   <bookViews>
-    <workbookView xWindow="6960" yWindow="1095" windowWidth="26730" windowHeight="18000" firstSheet="2" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="45435" yWindow="1845" windowWidth="26730" windowHeight="18000" firstSheet="2" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="14" r:id="rId1"/>
@@ -1008,22 +1008,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1066,12 +1050,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1124,12 +1102,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="26" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="29" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1254,6 +1226,34 @@
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1505,6 +1505,10 @@
     </sheetDataSet>
   </externalBook>
 </externalLink>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1844,23 +1848,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="A1" s="63" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" s="64"/>
-      <c r="C1" s="64"/>
-      <c r="D1" s="64"/>
-      <c r="E1" s="64"/>
-      <c r="F1" s="64"/>
-      <c r="G1" s="64"/>
-      <c r="H1" s="64"/>
-      <c r="I1" s="64"/>
-      <c r="J1" s="64"/>
-      <c r="K1" s="64"/>
-      <c r="L1" s="64"/>
-      <c r="M1" s="64"/>
-      <c r="N1" s="64"/>
-      <c r="O1" s="64"/>
+      <c r="A1" s="139" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="140"/>
+      <c r="C1" s="140"/>
+      <c r="D1" s="140"/>
+      <c r="E1" s="140"/>
+      <c r="F1" s="140"/>
+      <c r="G1" s="140"/>
+      <c r="H1" s="140"/>
+      <c r="I1" s="140"/>
+      <c r="J1" s="140"/>
+      <c r="K1" s="140"/>
+      <c r="L1" s="140"/>
+      <c r="M1" s="140"/>
+      <c r="N1" s="140"/>
+      <c r="O1" s="140"/>
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
       <c r="R1" s="1"/>
@@ -1874,23 +1878,23 @@
       <c r="Z1" s="1"/>
     </row>
     <row r="2" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A2" s="65" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="64"/>
-      <c r="C2" s="64"/>
-      <c r="D2" s="64"/>
-      <c r="E2" s="64"/>
-      <c r="F2" s="64"/>
-      <c r="G2" s="64"/>
-      <c r="H2" s="64"/>
-      <c r="I2" s="64"/>
-      <c r="J2" s="64"/>
-      <c r="K2" s="64"/>
-      <c r="L2" s="64"/>
-      <c r="M2" s="64"/>
-      <c r="N2" s="64"/>
-      <c r="O2" s="64"/>
+      <c r="A2" s="141" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="140"/>
+      <c r="C2" s="140"/>
+      <c r="D2" s="140"/>
+      <c r="E2" s="140"/>
+      <c r="F2" s="140"/>
+      <c r="G2" s="140"/>
+      <c r="H2" s="140"/>
+      <c r="I2" s="140"/>
+      <c r="J2" s="140"/>
+      <c r="K2" s="140"/>
+      <c r="L2" s="140"/>
+      <c r="M2" s="140"/>
+      <c r="N2" s="140"/>
+      <c r="O2" s="140"/>
       <c r="P2" s="1"/>
       <c r="Q2" s="1"/>
       <c r="R2" s="1"/>
@@ -2728,83 +2732,83 @@
     <col min="2" max="2" width="9.140625" style="62" bestFit="1" customWidth="1"/>
     <col min="3" max="11" width="10.7109375" style="62" customWidth="1"/>
     <col min="12" max="12" width="7.5703125" style="62" customWidth="1"/>
-    <col min="13" max="13" width="8.7109375" style="76" customWidth="1"/>
-    <col min="14" max="15" width="8.7109375" style="116" customWidth="1"/>
+    <col min="13" max="13" width="8.7109375" style="70" customWidth="1"/>
+    <col min="14" max="15" width="8.7109375" style="106" customWidth="1"/>
     <col min="16" max="23" width="8.7109375" style="62" customWidth="1"/>
     <col min="24" max="16384" width="14.140625" style="62"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" s="102" customFormat="1" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="105" t="s">
+    <row r="1" spans="1:23" s="94" customFormat="1" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="147" t="s">
         <v>56</v>
       </c>
-      <c r="B1" s="106"/>
-      <c r="C1" s="106"/>
-      <c r="D1" s="106"/>
-      <c r="E1" s="106"/>
-      <c r="F1" s="106"/>
-      <c r="G1" s="106"/>
-      <c r="H1" s="106"/>
-      <c r="I1" s="106"/>
-      <c r="J1" s="106"/>
-      <c r="K1" s="106"/>
-      <c r="L1" s="106"/>
-      <c r="M1" s="89" t="s">
+      <c r="B1" s="148"/>
+      <c r="C1" s="148"/>
+      <c r="D1" s="148"/>
+      <c r="E1" s="148"/>
+      <c r="F1" s="148"/>
+      <c r="G1" s="148"/>
+      <c r="H1" s="148"/>
+      <c r="I1" s="148"/>
+      <c r="J1" s="148"/>
+      <c r="K1" s="148"/>
+      <c r="L1" s="148"/>
+      <c r="M1" s="81" t="s">
         <v>54</v>
       </c>
-      <c r="N1" s="110"/>
-      <c r="O1" s="111" t="s">
+      <c r="N1" s="100"/>
+      <c r="O1" s="101" t="s">
         <v>55</v>
       </c>
-      <c r="P1" s="101"/>
-      <c r="Q1" s="101"/>
-      <c r="R1" s="101"/>
-      <c r="S1" s="101"/>
-      <c r="T1" s="101"/>
-      <c r="U1" s="101"/>
-      <c r="V1" s="101"/>
-      <c r="W1" s="101"/>
+      <c r="P1" s="93"/>
+      <c r="Q1" s="93"/>
+      <c r="R1" s="93"/>
+      <c r="S1" s="93"/>
+      <c r="T1" s="93"/>
+      <c r="U1" s="93"/>
+      <c r="V1" s="93"/>
+      <c r="W1" s="93"/>
     </row>
     <row r="2" spans="1:23" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="103" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" s="104" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" s="104">
-        <v>1</v>
-      </c>
-      <c r="D2" s="104">
-        <v>2</v>
-      </c>
-      <c r="E2" s="104">
-        <v>3</v>
-      </c>
-      <c r="F2" s="104">
-        <v>4</v>
-      </c>
-      <c r="G2" s="104">
-        <v>5</v>
-      </c>
-      <c r="H2" s="104">
-        <v>6</v>
-      </c>
-      <c r="I2" s="104">
+      <c r="A2" s="95" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="96" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="96">
+        <v>1</v>
+      </c>
+      <c r="D2" s="96">
+        <v>2</v>
+      </c>
+      <c r="E2" s="96">
+        <v>3</v>
+      </c>
+      <c r="F2" s="96">
+        <v>4</v>
+      </c>
+      <c r="G2" s="96">
+        <v>5</v>
+      </c>
+      <c r="H2" s="96">
+        <v>6</v>
+      </c>
+      <c r="I2" s="96">
         <v>7</v>
       </c>
-      <c r="J2" s="104">
+      <c r="J2" s="96">
         <v>8</v>
       </c>
-      <c r="K2" s="104">
+      <c r="K2" s="96">
         <v>9</v>
       </c>
-      <c r="L2" s="107" t="s">
+      <c r="L2" s="97" t="s">
         <v>7</v>
       </c>
-      <c r="M2" s="108"/>
-      <c r="N2" s="112"/>
-      <c r="O2" s="113"/>
+      <c r="M2" s="98"/>
+      <c r="N2" s="102"/>
+      <c r="O2" s="103"/>
       <c r="P2" s="3"/>
       <c r="Q2" s="3"/>
       <c r="R2" s="3"/>
@@ -2846,10 +2850,10 @@
       <c r="K3" s="6">
         <v>5</v>
       </c>
-      <c r="L3" s="79"/>
-      <c r="M3" s="109"/>
-      <c r="N3" s="114"/>
-      <c r="O3" s="115"/>
+      <c r="L3" s="73"/>
+      <c r="M3" s="99"/>
+      <c r="N3" s="104"/>
+      <c r="O3" s="105"/>
       <c r="P3" s="3"/>
       <c r="Q3" s="3"/>
       <c r="R3" s="3"/>
@@ -2891,10 +2895,10 @@
       <c r="K4" s="25">
         <v>2</v>
       </c>
-      <c r="L4" s="80"/>
-      <c r="M4" s="109"/>
-      <c r="N4" s="114"/>
-      <c r="O4" s="115"/>
+      <c r="L4" s="74"/>
+      <c r="M4" s="99"/>
+      <c r="N4" s="104"/>
+      <c r="O4" s="105"/>
       <c r="P4" s="3"/>
       <c r="Q4" s="3"/>
       <c r="R4" s="3"/>
@@ -2938,10 +2942,10 @@
       <c r="K5" s="12">
         <v>5</v>
       </c>
-      <c r="L5" s="81"/>
-      <c r="M5" s="117"/>
-      <c r="N5" s="118"/>
-      <c r="O5" s="144"/>
+      <c r="L5" s="75"/>
+      <c r="M5" s="107"/>
+      <c r="N5" s="108"/>
+      <c r="O5" s="134"/>
       <c r="P5" s="1"/>
       <c r="Q5" s="1"/>
       <c r="R5" s="1"/>
@@ -2952,44 +2956,44 @@
       <c r="W5" s="1"/>
     </row>
     <row r="6" spans="1:23" ht="15" x14ac:dyDescent="0.25">
-      <c r="A6" s="69"/>
-      <c r="B6" s="70" t="s">
+      <c r="A6" s="63"/>
+      <c r="B6" s="64" t="s">
         <v>40</v>
       </c>
-      <c r="C6" s="70">
-        <v>2</v>
-      </c>
-      <c r="D6" s="70">
-        <v>2</v>
-      </c>
-      <c r="E6" s="70">
-        <v>2</v>
-      </c>
-      <c r="F6" s="70">
-        <v>1</v>
-      </c>
-      <c r="G6" s="70">
-        <v>2</v>
-      </c>
-      <c r="H6" s="70">
-        <v>1</v>
-      </c>
-      <c r="I6" s="70">
-        <v>1</v>
-      </c>
-      <c r="J6" s="70">
-        <v>2</v>
-      </c>
-      <c r="K6" s="70">
-        <v>2</v>
-      </c>
-      <c r="L6" s="82">
+      <c r="C6" s="64">
+        <v>2</v>
+      </c>
+      <c r="D6" s="64">
+        <v>2</v>
+      </c>
+      <c r="E6" s="64">
+        <v>2</v>
+      </c>
+      <c r="F6" s="64">
+        <v>1</v>
+      </c>
+      <c r="G6" s="64">
+        <v>2</v>
+      </c>
+      <c r="H6" s="64">
+        <v>1</v>
+      </c>
+      <c r="I6" s="64">
+        <v>1</v>
+      </c>
+      <c r="J6" s="64">
+        <v>2</v>
+      </c>
+      <c r="K6" s="64">
+        <v>2</v>
+      </c>
+      <c r="L6" s="76">
         <f>SUM(C6:K6)</f>
         <v>15</v>
       </c>
-      <c r="M6" s="93"/>
-      <c r="N6" s="119"/>
-      <c r="O6" s="121"/>
+      <c r="M6" s="85"/>
+      <c r="N6" s="109"/>
+      <c r="O6" s="111"/>
       <c r="P6" s="1"/>
       <c r="Q6" s="1"/>
       <c r="R6" s="1"/>
@@ -3008,15 +3012,15 @@
         <f>C5-C6</f>
         <v>4</v>
       </c>
-      <c r="D7" s="73">
+      <c r="D7" s="67">
         <f t="shared" ref="D7:K7" si="0">D5-D6</f>
         <v>3</v>
       </c>
-      <c r="E7" s="73">
+      <c r="E7" s="67">
         <f t="shared" si="0"/>
         <v>2</v>
       </c>
-      <c r="F7" s="73">
+      <c r="F7" s="67">
         <f t="shared" si="0"/>
         <v>2</v>
       </c>
@@ -3036,18 +3040,18 @@
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="K7" s="73">
+      <c r="K7" s="67">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="L7" s="83"/>
-      <c r="M7" s="93">
+      <c r="L7" s="77"/>
+      <c r="M7" s="85">
         <v>2.5</v>
       </c>
-      <c r="N7" s="119">
+      <c r="N7" s="109">
         <v>8.33</v>
       </c>
-      <c r="O7" s="121">
+      <c r="O7" s="111">
         <v>8</v>
       </c>
       <c r="P7" s="1"/>
@@ -3093,10 +3097,10 @@
       <c r="K8" s="12">
         <v>6</v>
       </c>
-      <c r="L8" s="81"/>
-      <c r="M8" s="93"/>
-      <c r="N8" s="119"/>
-      <c r="O8" s="121"/>
+      <c r="L8" s="75"/>
+      <c r="M8" s="85"/>
+      <c r="N8" s="109"/>
+      <c r="O8" s="111"/>
       <c r="P8" s="1"/>
       <c r="Q8" s="1"/>
       <c r="R8" s="1"/>
@@ -3107,44 +3111,44 @@
       <c r="W8" s="1"/>
     </row>
     <row r="9" spans="1:23" ht="15" x14ac:dyDescent="0.25">
-      <c r="A9" s="69"/>
-      <c r="B9" s="70" t="s">
+      <c r="A9" s="63"/>
+      <c r="B9" s="64" t="s">
         <v>40</v>
       </c>
-      <c r="C9" s="70">
-        <v>3</v>
-      </c>
-      <c r="D9" s="70">
-        <v>3</v>
-      </c>
-      <c r="E9" s="70">
-        <v>3</v>
-      </c>
-      <c r="F9" s="70">
-        <v>2</v>
-      </c>
-      <c r="G9" s="70">
-        <v>2</v>
-      </c>
-      <c r="H9" s="70">
-        <v>2</v>
-      </c>
-      <c r="I9" s="70">
-        <v>2</v>
-      </c>
-      <c r="J9" s="70">
-        <v>2</v>
-      </c>
-      <c r="K9" s="70">
-        <v>3</v>
-      </c>
-      <c r="L9" s="82">
+      <c r="C9" s="64">
+        <v>3</v>
+      </c>
+      <c r="D9" s="64">
+        <v>3</v>
+      </c>
+      <c r="E9" s="64">
+        <v>3</v>
+      </c>
+      <c r="F9" s="64">
+        <v>2</v>
+      </c>
+      <c r="G9" s="64">
+        <v>2</v>
+      </c>
+      <c r="H9" s="64">
+        <v>2</v>
+      </c>
+      <c r="I9" s="64">
+        <v>2</v>
+      </c>
+      <c r="J9" s="64">
+        <v>2</v>
+      </c>
+      <c r="K9" s="64">
+        <v>3</v>
+      </c>
+      <c r="L9" s="76">
         <f>SUM(C9:K9)</f>
         <v>22</v>
       </c>
-      <c r="M9" s="93"/>
-      <c r="N9" s="119"/>
-      <c r="O9" s="121"/>
+      <c r="M9" s="85"/>
+      <c r="N9" s="109"/>
+      <c r="O9" s="111"/>
       <c r="P9" s="1"/>
       <c r="Q9" s="1"/>
       <c r="R9" s="1"/>
@@ -3159,7 +3163,7 @@
       <c r="B10" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="C10" s="73">
+      <c r="C10" s="67">
         <f>C8-C9</f>
         <v>2</v>
       </c>
@@ -3171,7 +3175,7 @@
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
-      <c r="F10" s="73">
+      <c r="F10" s="67">
         <f t="shared" si="1"/>
         <v>2</v>
       </c>
@@ -3187,22 +3191,22 @@
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
-      <c r="J10" s="73">
+      <c r="J10" s="67">
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
-      <c r="K10" s="73">
+      <c r="K10" s="67">
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
-      <c r="L10" s="83"/>
-      <c r="M10" s="93">
+      <c r="L10" s="77"/>
+      <c r="M10" s="85">
         <v>2.5</v>
       </c>
-      <c r="N10" s="119">
+      <c r="N10" s="109">
         <v>8.33</v>
       </c>
-      <c r="O10" s="121">
+      <c r="O10" s="111">
         <v>8</v>
       </c>
       <c r="P10" s="1"/>
@@ -3248,12 +3252,12 @@
       <c r="K11" s="12">
         <v>6</v>
       </c>
-      <c r="L11" s="81">
+      <c r="L11" s="75">
         <v>10</v>
       </c>
-      <c r="M11" s="93"/>
-      <c r="N11" s="119"/>
-      <c r="O11" s="121"/>
+      <c r="M11" s="85"/>
+      <c r="N11" s="109"/>
+      <c r="O11" s="111"/>
       <c r="P11" s="1"/>
       <c r="Q11" s="1"/>
       <c r="R11" s="1"/>
@@ -3264,41 +3268,41 @@
       <c r="W11" s="1"/>
     </row>
     <row r="12" spans="1:23" ht="15" x14ac:dyDescent="0.25">
-      <c r="A12" s="69"/>
-      <c r="B12" s="70" t="s">
+      <c r="A12" s="63"/>
+      <c r="B12" s="64" t="s">
         <v>40</v>
       </c>
-      <c r="C12" s="70">
-        <v>1</v>
-      </c>
-      <c r="D12" s="70">
-        <v>2</v>
-      </c>
-      <c r="E12" s="70">
-        <v>1</v>
-      </c>
-      <c r="F12" s="70">
-        <v>1</v>
-      </c>
-      <c r="G12" s="70">
-        <v>1</v>
-      </c>
-      <c r="H12" s="70">
-        <v>1</v>
-      </c>
-      <c r="I12" s="70">
-        <v>1</v>
-      </c>
-      <c r="J12" s="70">
-        <v>1</v>
-      </c>
-      <c r="K12" s="70">
-        <v>1</v>
-      </c>
-      <c r="L12" s="82"/>
-      <c r="M12" s="93"/>
-      <c r="N12" s="119"/>
-      <c r="O12" s="121"/>
+      <c r="C12" s="64">
+        <v>1</v>
+      </c>
+      <c r="D12" s="64">
+        <v>2</v>
+      </c>
+      <c r="E12" s="64">
+        <v>1</v>
+      </c>
+      <c r="F12" s="64">
+        <v>1</v>
+      </c>
+      <c r="G12" s="64">
+        <v>1</v>
+      </c>
+      <c r="H12" s="64">
+        <v>1</v>
+      </c>
+      <c r="I12" s="64">
+        <v>1</v>
+      </c>
+      <c r="J12" s="64">
+        <v>1</v>
+      </c>
+      <c r="K12" s="64">
+        <v>1</v>
+      </c>
+      <c r="L12" s="76"/>
+      <c r="M12" s="85"/>
+      <c r="N12" s="109"/>
+      <c r="O12" s="111"/>
       <c r="P12" s="1"/>
       <c r="Q12" s="1"/>
       <c r="R12" s="1"/>
@@ -3329,7 +3333,7 @@
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
-      <c r="G13" s="73">
+      <c r="G13" s="67">
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
@@ -3337,7 +3341,7 @@
         <f t="shared" si="2"/>
         <v>5</v>
       </c>
-      <c r="I13" s="73">
+      <c r="I13" s="67">
         <f t="shared" si="2"/>
         <v>2</v>
       </c>
@@ -3349,14 +3353,14 @@
         <f t="shared" si="2"/>
         <v>5</v>
       </c>
-      <c r="L13" s="83"/>
-      <c r="M13" s="93">
-        <v>1</v>
-      </c>
-      <c r="N13" s="119">
+      <c r="L13" s="77"/>
+      <c r="M13" s="85">
+        <v>1</v>
+      </c>
+      <c r="N13" s="109">
         <v>3.33</v>
       </c>
-      <c r="O13" s="121">
+      <c r="O13" s="111">
         <v>3</v>
       </c>
       <c r="P13" s="1"/>
@@ -3402,10 +3406,10 @@
       <c r="K14" s="12">
         <v>4</v>
       </c>
-      <c r="L14" s="81"/>
-      <c r="M14" s="93"/>
-      <c r="N14" s="119"/>
-      <c r="O14" s="121"/>
+      <c r="L14" s="75"/>
+      <c r="M14" s="85"/>
+      <c r="N14" s="109"/>
+      <c r="O14" s="111"/>
       <c r="P14" s="1"/>
       <c r="Q14" s="1"/>
       <c r="R14" s="1"/>
@@ -3416,44 +3420,44 @@
       <c r="W14" s="1"/>
     </row>
     <row r="15" spans="1:23" ht="15" x14ac:dyDescent="0.25">
-      <c r="A15" s="69"/>
-      <c r="B15" s="70" t="s">
+      <c r="A15" s="63"/>
+      <c r="B15" s="64" t="s">
         <v>40</v>
       </c>
-      <c r="C15" s="70">
-        <v>1</v>
-      </c>
-      <c r="D15" s="70">
-        <v>1</v>
-      </c>
-      <c r="E15" s="70">
-        <v>1</v>
-      </c>
-      <c r="F15" s="70">
+      <c r="C15" s="64">
+        <v>1</v>
+      </c>
+      <c r="D15" s="64">
+        <v>1</v>
+      </c>
+      <c r="E15" s="64">
+        <v>1</v>
+      </c>
+      <c r="F15" s="64">
         <v>0</v>
       </c>
-      <c r="G15" s="70">
-        <v>1</v>
-      </c>
-      <c r="H15" s="70">
-        <v>1</v>
-      </c>
-      <c r="I15" s="70">
-        <v>1</v>
-      </c>
-      <c r="J15" s="70">
-        <v>1</v>
-      </c>
-      <c r="K15" s="70">
-        <v>1</v>
-      </c>
-      <c r="L15" s="82">
+      <c r="G15" s="64">
+        <v>1</v>
+      </c>
+      <c r="H15" s="64">
+        <v>1</v>
+      </c>
+      <c r="I15" s="64">
+        <v>1</v>
+      </c>
+      <c r="J15" s="64">
+        <v>1</v>
+      </c>
+      <c r="K15" s="64">
+        <v>1</v>
+      </c>
+      <c r="L15" s="76">
         <f>SUM(C15:K15)</f>
         <v>8</v>
       </c>
-      <c r="M15" s="93"/>
-      <c r="N15" s="119"/>
-      <c r="O15" s="121"/>
+      <c r="M15" s="85"/>
+      <c r="N15" s="109"/>
+      <c r="O15" s="111"/>
       <c r="P15" s="1"/>
       <c r="Q15" s="1"/>
       <c r="R15" s="1"/>
@@ -3488,7 +3492,7 @@
         <f t="shared" si="3"/>
         <v>5</v>
       </c>
-      <c r="H16" s="73">
+      <c r="H16" s="67">
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
@@ -3500,18 +3504,18 @@
         <f t="shared" si="3"/>
         <v>4</v>
       </c>
-      <c r="K16" s="73">
+      <c r="K16" s="67">
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
-      <c r="L16" s="83"/>
-      <c r="M16" s="93">
-        <v>1</v>
-      </c>
-      <c r="N16" s="119">
+      <c r="L16" s="77"/>
+      <c r="M16" s="85">
+        <v>1</v>
+      </c>
+      <c r="N16" s="109">
         <v>3.33</v>
       </c>
-      <c r="O16" s="121">
+      <c r="O16" s="111">
         <v>3</v>
       </c>
       <c r="P16" s="1"/>
@@ -3557,10 +3561,10 @@
       <c r="K17" s="12">
         <v>4</v>
       </c>
-      <c r="L17" s="81"/>
-      <c r="M17" s="93"/>
-      <c r="N17" s="119"/>
-      <c r="O17" s="121"/>
+      <c r="L17" s="75"/>
+      <c r="M17" s="85"/>
+      <c r="N17" s="109"/>
+      <c r="O17" s="111"/>
       <c r="P17" s="1"/>
       <c r="Q17" s="1"/>
       <c r="R17" s="1"/>
@@ -3571,44 +3575,44 @@
       <c r="W17" s="1"/>
     </row>
     <row r="18" spans="1:23" ht="15" x14ac:dyDescent="0.25">
-      <c r="A18" s="69"/>
-      <c r="B18" s="70" t="s">
+      <c r="A18" s="63"/>
+      <c r="B18" s="64" t="s">
         <v>40</v>
       </c>
-      <c r="C18" s="70">
-        <v>1</v>
-      </c>
-      <c r="D18" s="70">
-        <v>1</v>
-      </c>
-      <c r="E18" s="70">
-        <v>1</v>
-      </c>
-      <c r="F18" s="70">
+      <c r="C18" s="64">
+        <v>1</v>
+      </c>
+      <c r="D18" s="64">
+        <v>1</v>
+      </c>
+      <c r="E18" s="64">
+        <v>1</v>
+      </c>
+      <c r="F18" s="64">
         <v>0</v>
       </c>
-      <c r="G18" s="70">
-        <v>1</v>
-      </c>
-      <c r="H18" s="70">
-        <v>1</v>
-      </c>
-      <c r="I18" s="70">
-        <v>1</v>
-      </c>
-      <c r="J18" s="70">
-        <v>1</v>
-      </c>
-      <c r="K18" s="70">
-        <v>1</v>
-      </c>
-      <c r="L18" s="82">
+      <c r="G18" s="64">
+        <v>1</v>
+      </c>
+      <c r="H18" s="64">
+        <v>1</v>
+      </c>
+      <c r="I18" s="64">
+        <v>1</v>
+      </c>
+      <c r="J18" s="64">
+        <v>1</v>
+      </c>
+      <c r="K18" s="64">
+        <v>1</v>
+      </c>
+      <c r="L18" s="76">
         <f>SUM(C18:K18)</f>
         <v>8</v>
       </c>
-      <c r="M18" s="93"/>
-      <c r="N18" s="119"/>
-      <c r="O18" s="121"/>
+      <c r="M18" s="85"/>
+      <c r="N18" s="109"/>
+      <c r="O18" s="111"/>
       <c r="P18" s="1"/>
       <c r="Q18" s="1"/>
       <c r="R18" s="1"/>
@@ -3647,26 +3651,26 @@
         <f t="shared" si="4"/>
         <v>5</v>
       </c>
-      <c r="I19" s="73">
+      <c r="I19" s="67">
         <f t="shared" si="4"/>
         <v>2</v>
       </c>
-      <c r="J19" s="73">
+      <c r="J19" s="67">
         <f t="shared" si="4"/>
         <v>3</v>
       </c>
-      <c r="K19" s="73">
+      <c r="K19" s="67">
         <f t="shared" si="4"/>
         <v>3</v>
       </c>
-      <c r="L19" s="83"/>
-      <c r="M19" s="93">
-        <v>1</v>
-      </c>
-      <c r="N19" s="119">
+      <c r="L19" s="77"/>
+      <c r="M19" s="85">
+        <v>1</v>
+      </c>
+      <c r="N19" s="109">
         <v>3.33</v>
       </c>
-      <c r="O19" s="121">
+      <c r="O19" s="111">
         <v>3</v>
       </c>
       <c r="P19" s="1"/>
@@ -3712,10 +3716,10 @@
       <c r="K20" s="12">
         <v>8</v>
       </c>
-      <c r="L20" s="81"/>
-      <c r="M20" s="93"/>
-      <c r="N20" s="119"/>
-      <c r="O20" s="121"/>
+      <c r="L20" s="75"/>
+      <c r="M20" s="85"/>
+      <c r="N20" s="109"/>
+      <c r="O20" s="111"/>
       <c r="P20" s="1"/>
       <c r="Q20" s="1"/>
       <c r="R20" s="1"/>
@@ -3726,44 +3730,44 @@
       <c r="W20" s="1"/>
     </row>
     <row r="21" spans="1:23" ht="15" x14ac:dyDescent="0.25">
-      <c r="A21" s="69"/>
-      <c r="B21" s="70" t="s">
+      <c r="A21" s="63"/>
+      <c r="B21" s="64" t="s">
         <v>40</v>
       </c>
-      <c r="C21" s="70">
-        <v>2</v>
-      </c>
-      <c r="D21" s="70">
-        <v>2</v>
-      </c>
-      <c r="E21" s="70">
-        <v>2</v>
-      </c>
-      <c r="F21" s="70">
-        <v>1</v>
-      </c>
-      <c r="G21" s="70">
-        <v>2</v>
-      </c>
-      <c r="H21" s="70">
-        <v>2</v>
-      </c>
-      <c r="I21" s="70">
-        <v>2</v>
-      </c>
-      <c r="J21" s="70">
-        <v>2</v>
-      </c>
-      <c r="K21" s="70">
-        <v>2</v>
-      </c>
-      <c r="L21" s="82">
+      <c r="C21" s="64">
+        <v>2</v>
+      </c>
+      <c r="D21" s="64">
+        <v>2</v>
+      </c>
+      <c r="E21" s="64">
+        <v>2</v>
+      </c>
+      <c r="F21" s="64">
+        <v>1</v>
+      </c>
+      <c r="G21" s="64">
+        <v>2</v>
+      </c>
+      <c r="H21" s="64">
+        <v>2</v>
+      </c>
+      <c r="I21" s="64">
+        <v>2</v>
+      </c>
+      <c r="J21" s="64">
+        <v>2</v>
+      </c>
+      <c r="K21" s="64">
+        <v>2</v>
+      </c>
+      <c r="L21" s="76">
         <f>SUM(C21:K21)</f>
         <v>17</v>
       </c>
-      <c r="M21" s="93"/>
-      <c r="N21" s="119"/>
-      <c r="O21" s="121"/>
+      <c r="M21" s="85"/>
+      <c r="N21" s="109"/>
+      <c r="O21" s="111"/>
       <c r="P21" s="1"/>
       <c r="Q21" s="1"/>
       <c r="R21" s="1"/>
@@ -3802,7 +3806,7 @@
         <f t="shared" si="5"/>
         <v>5</v>
       </c>
-      <c r="I22" s="73">
+      <c r="I22" s="67">
         <f t="shared" si="5"/>
         <v>2</v>
       </c>
@@ -3814,14 +3818,14 @@
         <f t="shared" si="5"/>
         <v>6</v>
       </c>
-      <c r="L22" s="83"/>
-      <c r="M22" s="94">
+      <c r="L22" s="77"/>
+      <c r="M22" s="86">
         <v>0</v>
       </c>
-      <c r="N22" s="120">
+      <c r="N22" s="110">
         <v>0</v>
       </c>
-      <c r="O22" s="145"/>
+      <c r="O22" s="135"/>
       <c r="P22" s="1"/>
       <c r="Q22" s="1"/>
       <c r="R22" s="1"/>
@@ -3832,7 +3836,7 @@
       <c r="W22" s="1"/>
     </row>
     <row r="23" spans="1:23" ht="15" x14ac:dyDescent="0.25">
-      <c r="O23" s="146"/>
+      <c r="O23" s="136"/>
     </row>
     <row r="24" spans="1:23" ht="15" x14ac:dyDescent="0.25">
       <c r="C24" s="62" t="s">
@@ -3862,11 +3866,11 @@
       <c r="K24" s="62" t="s">
         <v>69</v>
       </c>
-      <c r="N24" s="116">
+      <c r="N24" s="106">
         <f>SUM(N7:N23)</f>
         <v>26.65</v>
       </c>
-      <c r="O24" s="146">
+      <c r="O24" s="136">
         <f>SUM(O7:O23)</f>
         <v>25</v>
       </c>
@@ -3905,23 +3909,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="A1" s="63" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" s="64"/>
-      <c r="C1" s="64"/>
-      <c r="D1" s="64"/>
-      <c r="E1" s="64"/>
-      <c r="F1" s="64"/>
-      <c r="G1" s="64"/>
-      <c r="H1" s="64"/>
-      <c r="I1" s="64"/>
-      <c r="J1" s="64"/>
-      <c r="K1" s="64"/>
-      <c r="L1" s="64"/>
-      <c r="M1" s="64"/>
-      <c r="N1" s="64"/>
-      <c r="O1" s="64"/>
+      <c r="A1" s="139" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="140"/>
+      <c r="C1" s="140"/>
+      <c r="D1" s="140"/>
+      <c r="E1" s="140"/>
+      <c r="F1" s="140"/>
+      <c r="G1" s="140"/>
+      <c r="H1" s="140"/>
+      <c r="I1" s="140"/>
+      <c r="J1" s="140"/>
+      <c r="K1" s="140"/>
+      <c r="L1" s="140"/>
+      <c r="M1" s="140"/>
+      <c r="N1" s="140"/>
+      <c r="O1" s="140"/>
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
       <c r="R1" s="1"/>
@@ -3935,23 +3939,23 @@
       <c r="Z1" s="1"/>
     </row>
     <row r="2" spans="1:26" ht="15" x14ac:dyDescent="0.25">
-      <c r="A2" s="65" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="64"/>
-      <c r="C2" s="64"/>
-      <c r="D2" s="64"/>
-      <c r="E2" s="64"/>
-      <c r="F2" s="64"/>
-      <c r="G2" s="64"/>
-      <c r="H2" s="64"/>
-      <c r="I2" s="64"/>
-      <c r="J2" s="64"/>
-      <c r="K2" s="64"/>
-      <c r="L2" s="64"/>
-      <c r="M2" s="64"/>
-      <c r="N2" s="64"/>
-      <c r="O2" s="64"/>
+      <c r="A2" s="141" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="140"/>
+      <c r="C2" s="140"/>
+      <c r="D2" s="140"/>
+      <c r="E2" s="140"/>
+      <c r="F2" s="140"/>
+      <c r="G2" s="140"/>
+      <c r="H2" s="140"/>
+      <c r="I2" s="140"/>
+      <c r="J2" s="140"/>
+      <c r="K2" s="140"/>
+      <c r="L2" s="140"/>
+      <c r="M2" s="140"/>
+      <c r="N2" s="140"/>
+      <c r="O2" s="140"/>
       <c r="P2" s="1"/>
       <c r="Q2" s="1"/>
       <c r="R2" s="1"/>
@@ -5787,81 +5791,81 @@
     <col min="9" max="9" width="11.85546875" style="62" customWidth="1"/>
     <col min="10" max="11" width="10.7109375" style="62" customWidth="1"/>
     <col min="12" max="12" width="7.42578125" style="62" customWidth="1"/>
-    <col min="13" max="13" width="7.42578125" style="139" customWidth="1"/>
+    <col min="13" max="13" width="7.42578125" style="129" customWidth="1"/>
     <col min="14" max="15" width="8.7109375" style="29" customWidth="1"/>
     <col min="16" max="23" width="8.7109375" style="62" customWidth="1"/>
     <col min="24" max="16384" width="14.140625" style="62"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" s="102" customFormat="1" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="105" t="s">
+    <row r="1" spans="1:23" s="94" customFormat="1" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="147" t="s">
         <v>71</v>
       </c>
-      <c r="B1" s="106"/>
-      <c r="C1" s="106"/>
-      <c r="D1" s="106"/>
-      <c r="E1" s="106"/>
-      <c r="F1" s="106"/>
-      <c r="G1" s="106"/>
-      <c r="H1" s="106"/>
-      <c r="I1" s="106"/>
-      <c r="J1" s="106"/>
-      <c r="K1" s="106"/>
-      <c r="L1" s="124"/>
-      <c r="M1" s="122" t="s">
+      <c r="B1" s="148"/>
+      <c r="C1" s="148"/>
+      <c r="D1" s="148"/>
+      <c r="E1" s="148"/>
+      <c r="F1" s="148"/>
+      <c r="G1" s="148"/>
+      <c r="H1" s="148"/>
+      <c r="I1" s="148"/>
+      <c r="J1" s="148"/>
+      <c r="K1" s="148"/>
+      <c r="L1" s="114"/>
+      <c r="M1" s="112" t="s">
         <v>54</v>
       </c>
-      <c r="N1" s="123"/>
-      <c r="O1" s="90" t="s">
+      <c r="N1" s="113"/>
+      <c r="O1" s="82" t="s">
         <v>55</v>
       </c>
-      <c r="P1" s="101"/>
-      <c r="Q1" s="101"/>
-      <c r="R1" s="101"/>
-      <c r="S1" s="101"/>
-      <c r="T1" s="101"/>
-      <c r="U1" s="101"/>
-      <c r="V1" s="101"/>
-      <c r="W1" s="101"/>
+      <c r="P1" s="93"/>
+      <c r="Q1" s="93"/>
+      <c r="R1" s="93"/>
+      <c r="S1" s="93"/>
+      <c r="T1" s="93"/>
+      <c r="U1" s="93"/>
+      <c r="V1" s="93"/>
+      <c r="W1" s="93"/>
     </row>
     <row r="2" spans="1:23" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="103" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" s="104" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" s="104">
-        <v>1</v>
-      </c>
-      <c r="D2" s="104">
-        <v>2</v>
-      </c>
-      <c r="E2" s="104">
-        <v>3</v>
-      </c>
-      <c r="F2" s="104">
-        <v>4</v>
-      </c>
-      <c r="G2" s="104">
-        <v>5</v>
-      </c>
-      <c r="H2" s="104">
-        <v>6</v>
-      </c>
-      <c r="I2" s="104">
+      <c r="A2" s="95" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="96" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="96">
+        <v>1</v>
+      </c>
+      <c r="D2" s="96">
+        <v>2</v>
+      </c>
+      <c r="E2" s="96">
+        <v>3</v>
+      </c>
+      <c r="F2" s="96">
+        <v>4</v>
+      </c>
+      <c r="G2" s="96">
+        <v>5</v>
+      </c>
+      <c r="H2" s="96">
+        <v>6</v>
+      </c>
+      <c r="I2" s="96">
         <v>7</v>
       </c>
-      <c r="J2" s="104">
+      <c r="J2" s="96">
         <v>8</v>
       </c>
-      <c r="K2" s="107">
+      <c r="K2" s="97">
         <v>9</v>
       </c>
-      <c r="L2" s="125"/>
-      <c r="M2" s="131"/>
-      <c r="N2" s="140"/>
-      <c r="O2" s="132"/>
+      <c r="L2" s="115"/>
+      <c r="M2" s="121"/>
+      <c r="N2" s="130"/>
+      <c r="O2" s="122"/>
       <c r="P2" s="3"/>
       <c r="Q2" s="3"/>
       <c r="R2" s="3"/>
@@ -5900,13 +5904,13 @@
       <c r="J3" s="6">
         <v>4</v>
       </c>
-      <c r="K3" s="79">
-        <v>5</v>
-      </c>
-      <c r="L3" s="126"/>
-      <c r="M3" s="133"/>
-      <c r="N3" s="134"/>
-      <c r="O3" s="134"/>
+      <c r="K3" s="73">
+        <v>5</v>
+      </c>
+      <c r="L3" s="116"/>
+      <c r="M3" s="123"/>
+      <c r="N3" s="124"/>
+      <c r="O3" s="124"/>
       <c r="P3" s="3"/>
       <c r="Q3" s="3"/>
       <c r="R3" s="3"/>
@@ -5945,13 +5949,13 @@
       <c r="J4" s="25">
         <v>6</v>
       </c>
-      <c r="K4" s="80">
-        <v>2</v>
-      </c>
-      <c r="L4" s="127"/>
-      <c r="M4" s="133"/>
-      <c r="N4" s="134"/>
-      <c r="O4" s="134"/>
+      <c r="K4" s="74">
+        <v>2</v>
+      </c>
+      <c r="L4" s="117"/>
+      <c r="M4" s="123"/>
+      <c r="N4" s="124"/>
+      <c r="O4" s="124"/>
       <c r="P4" s="3"/>
       <c r="Q4" s="3"/>
       <c r="R4" s="3"/>
@@ -5990,13 +5994,13 @@
       <c r="J5" s="12">
         <v>7</v>
       </c>
-      <c r="K5" s="81">
-        <v>4</v>
-      </c>
-      <c r="L5" s="128"/>
-      <c r="M5" s="135"/>
-      <c r="N5" s="136"/>
-      <c r="O5" s="136"/>
+      <c r="K5" s="75">
+        <v>4</v>
+      </c>
+      <c r="L5" s="118"/>
+      <c r="M5" s="125"/>
+      <c r="N5" s="126"/>
+      <c r="O5" s="126"/>
       <c r="P5" s="1"/>
       <c r="Q5" s="1"/>
       <c r="R5" s="1"/>
@@ -6006,43 +6010,43 @@
       <c r="V5" s="1"/>
       <c r="W5" s="1"/>
     </row>
-    <row r="6" spans="1:23" s="62" customFormat="1" ht="15" x14ac:dyDescent="0.25">
-      <c r="A6" s="69"/>
-      <c r="B6" s="70"/>
-      <c r="C6" s="70">
-        <v>2</v>
-      </c>
-      <c r="D6" s="70">
-        <v>2</v>
-      </c>
-      <c r="E6" s="70">
-        <v>2</v>
-      </c>
-      <c r="F6" s="70">
-        <v>1</v>
-      </c>
-      <c r="G6" s="70">
-        <v>1</v>
-      </c>
-      <c r="H6" s="70">
-        <v>1</v>
-      </c>
-      <c r="I6" s="70">
-        <v>1</v>
-      </c>
-      <c r="J6" s="70">
-        <v>1</v>
-      </c>
-      <c r="K6" s="82">
-        <v>2</v>
-      </c>
-      <c r="L6" s="128">
+    <row r="6" spans="1:23" ht="15" x14ac:dyDescent="0.25">
+      <c r="A6" s="63"/>
+      <c r="B6" s="64"/>
+      <c r="C6" s="64">
+        <v>2</v>
+      </c>
+      <c r="D6" s="64">
+        <v>2</v>
+      </c>
+      <c r="E6" s="64">
+        <v>2</v>
+      </c>
+      <c r="F6" s="64">
+        <v>1</v>
+      </c>
+      <c r="G6" s="64">
+        <v>1</v>
+      </c>
+      <c r="H6" s="64">
+        <v>1</v>
+      </c>
+      <c r="I6" s="64">
+        <v>1</v>
+      </c>
+      <c r="J6" s="64">
+        <v>1</v>
+      </c>
+      <c r="K6" s="76">
+        <v>2</v>
+      </c>
+      <c r="L6" s="118">
         <f>SUM(C6:K6)</f>
         <v>13</v>
       </c>
-      <c r="M6" s="135"/>
-      <c r="N6" s="136"/>
-      <c r="O6" s="136"/>
+      <c r="M6" s="125"/>
+      <c r="N6" s="126"/>
+      <c r="O6" s="126"/>
       <c r="P6" s="1"/>
       <c r="Q6" s="1"/>
       <c r="R6" s="1"/>
@@ -6055,19 +6059,19 @@
     <row r="7" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="15"/>
       <c r="B7" s="16"/>
-      <c r="C7" s="73">
+      <c r="C7" s="67">
         <f>C5-C6</f>
         <v>3</v>
       </c>
-      <c r="D7" s="73">
+      <c r="D7" s="67">
         <f t="shared" ref="D7:K7" si="0">D5-D6</f>
         <v>4</v>
       </c>
-      <c r="E7" s="73">
+      <c r="E7" s="67">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="F7" s="73">
+      <c r="F7" s="67">
         <f t="shared" si="0"/>
         <v>2</v>
       </c>
@@ -6087,18 +6091,18 @@
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="K7" s="130">
+      <c r="K7" s="120">
         <f t="shared" si="0"/>
         <v>2</v>
       </c>
-      <c r="L7" s="128"/>
-      <c r="M7" s="135">
+      <c r="L7" s="118"/>
+      <c r="M7" s="125">
         <v>2.5</v>
       </c>
-      <c r="N7" s="136">
+      <c r="N7" s="126">
         <v>11.1</v>
       </c>
-      <c r="O7" s="134">
+      <c r="O7" s="124">
         <v>11</v>
       </c>
       <c r="P7" s="1"/>
@@ -6139,13 +6143,13 @@
       <c r="J8" s="12">
         <v>6</v>
       </c>
-      <c r="K8" s="81">
+      <c r="K8" s="75">
         <v>7</v>
       </c>
-      <c r="L8" s="128"/>
-      <c r="M8" s="135"/>
-      <c r="N8" s="136"/>
-      <c r="O8" s="134"/>
+      <c r="L8" s="118"/>
+      <c r="M8" s="125"/>
+      <c r="N8" s="126"/>
+      <c r="O8" s="124"/>
       <c r="P8" s="1"/>
       <c r="Q8" s="1"/>
       <c r="R8" s="1"/>
@@ -6155,43 +6159,43 @@
       <c r="V8" s="1"/>
       <c r="W8" s="1"/>
     </row>
-    <row r="9" spans="1:23" s="62" customFormat="1" ht="15" x14ac:dyDescent="0.25">
-      <c r="A9" s="69"/>
-      <c r="B9" s="70"/>
-      <c r="C9" s="70">
-        <v>2</v>
-      </c>
-      <c r="D9" s="70">
-        <v>2</v>
-      </c>
-      <c r="E9" s="70">
-        <v>2</v>
-      </c>
-      <c r="F9" s="70">
-        <v>1</v>
-      </c>
-      <c r="G9" s="70">
-        <v>1</v>
-      </c>
-      <c r="H9" s="70">
-        <v>1</v>
-      </c>
-      <c r="I9" s="70">
-        <v>1</v>
-      </c>
-      <c r="J9" s="70">
-        <v>1</v>
-      </c>
-      <c r="K9" s="82">
-        <v>2</v>
-      </c>
-      <c r="L9" s="128">
+    <row r="9" spans="1:23" ht="15" x14ac:dyDescent="0.25">
+      <c r="A9" s="63"/>
+      <c r="B9" s="64"/>
+      <c r="C9" s="64">
+        <v>2</v>
+      </c>
+      <c r="D9" s="64">
+        <v>2</v>
+      </c>
+      <c r="E9" s="64">
+        <v>2</v>
+      </c>
+      <c r="F9" s="64">
+        <v>1</v>
+      </c>
+      <c r="G9" s="64">
+        <v>1</v>
+      </c>
+      <c r="H9" s="64">
+        <v>1</v>
+      </c>
+      <c r="I9" s="64">
+        <v>1</v>
+      </c>
+      <c r="J9" s="64">
+        <v>1</v>
+      </c>
+      <c r="K9" s="76">
+        <v>2</v>
+      </c>
+      <c r="L9" s="118">
         <f>SUM(C9:K9)</f>
         <v>13</v>
       </c>
-      <c r="M9" s="135"/>
-      <c r="N9" s="136"/>
-      <c r="O9" s="134"/>
+      <c r="M9" s="125"/>
+      <c r="N9" s="126"/>
+      <c r="O9" s="124"/>
       <c r="P9" s="1"/>
       <c r="Q9" s="1"/>
       <c r="R9" s="1"/>
@@ -6212,7 +6216,7 @@
         <f t="shared" ref="D10:K10" si="1">D8-D9</f>
         <v>4</v>
       </c>
-      <c r="E10" s="73">
+      <c r="E10" s="67">
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
@@ -6224,11 +6228,11 @@
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
-      <c r="H10" s="73">
+      <c r="H10" s="67">
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
-      <c r="I10" s="73">
+      <c r="I10" s="67">
         <f t="shared" si="1"/>
         <v>2</v>
       </c>
@@ -6236,18 +6240,18 @@
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="K10" s="83">
+      <c r="K10" s="77">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L10" s="128"/>
-      <c r="M10" s="135">
+      <c r="L10" s="118"/>
+      <c r="M10" s="125">
         <v>2.5</v>
       </c>
-      <c r="N10" s="136">
+      <c r="N10" s="126">
         <v>11.1</v>
       </c>
-      <c r="O10" s="134">
+      <c r="O10" s="124">
         <v>11</v>
       </c>
       <c r="P10" s="1"/>
@@ -6288,13 +6292,13 @@
       <c r="J11" s="12">
         <v>4</v>
       </c>
-      <c r="K11" s="81">
-        <v>6</v>
-      </c>
-      <c r="L11" s="128"/>
-      <c r="M11" s="135"/>
-      <c r="N11" s="136"/>
-      <c r="O11" s="134"/>
+      <c r="K11" s="75">
+        <v>6</v>
+      </c>
+      <c r="L11" s="118"/>
+      <c r="M11" s="125"/>
+      <c r="N11" s="126"/>
+      <c r="O11" s="124"/>
       <c r="P11" s="1"/>
       <c r="Q11" s="1"/>
       <c r="R11" s="1"/>
@@ -6304,43 +6308,43 @@
       <c r="V11" s="1"/>
       <c r="W11" s="1"/>
     </row>
-    <row r="12" spans="1:23" s="62" customFormat="1" ht="15" x14ac:dyDescent="0.25">
-      <c r="A12" s="69"/>
-      <c r="B12" s="70"/>
-      <c r="C12" s="70">
-        <v>1</v>
-      </c>
-      <c r="D12" s="70">
-        <v>1</v>
-      </c>
-      <c r="E12" s="70">
-        <v>1</v>
-      </c>
-      <c r="F12" s="70">
+    <row r="12" spans="1:23" ht="15" x14ac:dyDescent="0.25">
+      <c r="A12" s="63"/>
+      <c r="B12" s="64"/>
+      <c r="C12" s="64">
+        <v>1</v>
+      </c>
+      <c r="D12" s="64">
+        <v>1</v>
+      </c>
+      <c r="E12" s="64">
+        <v>1</v>
+      </c>
+      <c r="F12" s="64">
         <v>0</v>
       </c>
-      <c r="G12" s="70">
-        <v>1</v>
-      </c>
-      <c r="H12" s="70">
-        <v>1</v>
-      </c>
-      <c r="I12" s="70">
-        <v>1</v>
-      </c>
-      <c r="J12" s="70">
-        <v>1</v>
-      </c>
-      <c r="K12" s="82">
-        <v>1</v>
-      </c>
-      <c r="L12" s="128">
+      <c r="G12" s="64">
+        <v>1</v>
+      </c>
+      <c r="H12" s="64">
+        <v>1</v>
+      </c>
+      <c r="I12" s="64">
+        <v>1</v>
+      </c>
+      <c r="J12" s="64">
+        <v>1</v>
+      </c>
+      <c r="K12" s="76">
+        <v>1</v>
+      </c>
+      <c r="L12" s="118">
         <f>SUM(C12:K12)</f>
         <v>8</v>
       </c>
-      <c r="M12" s="135"/>
-      <c r="N12" s="136"/>
-      <c r="O12" s="134"/>
+      <c r="M12" s="125"/>
+      <c r="N12" s="126"/>
+      <c r="O12" s="124"/>
       <c r="P12" s="1"/>
       <c r="Q12" s="1"/>
       <c r="R12" s="1"/>
@@ -6353,7 +6357,7 @@
     <row r="13" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="15"/>
       <c r="B13" s="16"/>
-      <c r="C13" s="73">
+      <c r="C13" s="67">
         <f>C11-C12</f>
         <v>3</v>
       </c>
@@ -6373,7 +6377,7 @@
         <f t="shared" si="2"/>
         <v>4</v>
       </c>
-      <c r="H13" s="73">
+      <c r="H13" s="67">
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
@@ -6381,22 +6385,22 @@
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
-      <c r="J13" s="73">
+      <c r="J13" s="67">
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
-      <c r="K13" s="83">
+      <c r="K13" s="77">
         <f t="shared" si="2"/>
         <v>5</v>
       </c>
-      <c r="L13" s="128"/>
-      <c r="M13" s="135">
-        <v>1</v>
-      </c>
-      <c r="N13" s="136">
+      <c r="L13" s="118"/>
+      <c r="M13" s="125">
+        <v>1</v>
+      </c>
+      <c r="N13" s="126">
         <v>4.4400000000000004</v>
       </c>
-      <c r="O13" s="134">
+      <c r="O13" s="124">
         <v>4</v>
       </c>
       <c r="P13" s="1"/>
@@ -6437,13 +6441,13 @@
       <c r="J14" s="12">
         <v>5</v>
       </c>
-      <c r="K14" s="81">
-        <v>6</v>
-      </c>
-      <c r="L14" s="128"/>
-      <c r="M14" s="135"/>
-      <c r="N14" s="136"/>
-      <c r="O14" s="134"/>
+      <c r="K14" s="75">
+        <v>6</v>
+      </c>
+      <c r="L14" s="118"/>
+      <c r="M14" s="125"/>
+      <c r="N14" s="126"/>
+      <c r="O14" s="124"/>
       <c r="P14" s="1"/>
       <c r="Q14" s="1"/>
       <c r="R14" s="1"/>
@@ -6453,43 +6457,43 @@
       <c r="V14" s="1"/>
       <c r="W14" s="1"/>
     </row>
-    <row r="15" spans="1:23" s="62" customFormat="1" ht="15" x14ac:dyDescent="0.25">
-      <c r="A15" s="69"/>
-      <c r="B15" s="70"/>
-      <c r="C15" s="70">
-        <v>2</v>
-      </c>
-      <c r="D15" s="70">
-        <v>2</v>
-      </c>
-      <c r="E15" s="70">
-        <v>2</v>
-      </c>
-      <c r="F15" s="70">
-        <v>1</v>
-      </c>
-      <c r="G15" s="70">
-        <v>2</v>
-      </c>
-      <c r="H15" s="70">
-        <v>1</v>
-      </c>
-      <c r="I15" s="70">
-        <v>1</v>
-      </c>
-      <c r="J15" s="70">
-        <v>2</v>
-      </c>
-      <c r="K15" s="82">
-        <v>2</v>
-      </c>
-      <c r="L15" s="128">
+    <row r="15" spans="1:23" ht="15" x14ac:dyDescent="0.25">
+      <c r="A15" s="63"/>
+      <c r="B15" s="64"/>
+      <c r="C15" s="64">
+        <v>2</v>
+      </c>
+      <c r="D15" s="64">
+        <v>2</v>
+      </c>
+      <c r="E15" s="64">
+        <v>2</v>
+      </c>
+      <c r="F15" s="64">
+        <v>1</v>
+      </c>
+      <c r="G15" s="64">
+        <v>2</v>
+      </c>
+      <c r="H15" s="64">
+        <v>1</v>
+      </c>
+      <c r="I15" s="64">
+        <v>1</v>
+      </c>
+      <c r="J15" s="64">
+        <v>2</v>
+      </c>
+      <c r="K15" s="76">
+        <v>2</v>
+      </c>
+      <c r="L15" s="118">
         <f>SUM(C15:K15)</f>
         <v>15</v>
       </c>
-      <c r="M15" s="135"/>
-      <c r="N15" s="136"/>
-      <c r="O15" s="134"/>
+      <c r="M15" s="125"/>
+      <c r="N15" s="126"/>
+      <c r="O15" s="124"/>
       <c r="P15" s="1"/>
       <c r="Q15" s="1"/>
       <c r="R15" s="1"/>
@@ -6502,11 +6506,11 @@
     <row r="16" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="15"/>
       <c r="B16" s="16"/>
-      <c r="C16" s="73">
+      <c r="C16" s="67">
         <f>C14-C15</f>
         <v>3</v>
       </c>
-      <c r="D16" s="73">
+      <c r="D16" s="67">
         <f t="shared" ref="D16:K16" si="3">D14-D15</f>
         <v>4</v>
       </c>
@@ -6514,7 +6518,7 @@
         <f t="shared" si="3"/>
         <v>4</v>
       </c>
-      <c r="F16" s="73">
+      <c r="F16" s="67">
         <f t="shared" si="3"/>
         <v>2</v>
       </c>
@@ -6530,22 +6534,22 @@
         <f t="shared" si="3"/>
         <v>4</v>
       </c>
-      <c r="J16" s="73">
+      <c r="J16" s="67">
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
-      <c r="K16" s="83">
+      <c r="K16" s="77">
         <f t="shared" si="3"/>
         <v>4</v>
       </c>
-      <c r="L16" s="128"/>
-      <c r="M16" s="135">
+      <c r="L16" s="118"/>
+      <c r="M16" s="125">
         <v>0.5</v>
       </c>
-      <c r="N16" s="136">
+      <c r="N16" s="126">
         <v>2.2200000000000002</v>
       </c>
-      <c r="O16" s="134">
+      <c r="O16" s="124">
         <v>2</v>
       </c>
       <c r="P16" s="1"/>
@@ -6586,13 +6590,13 @@
       <c r="J17" s="12">
         <v>5</v>
       </c>
-      <c r="K17" s="81">
-        <v>6</v>
-      </c>
-      <c r="L17" s="128"/>
-      <c r="M17" s="135"/>
-      <c r="N17" s="136"/>
-      <c r="O17" s="134"/>
+      <c r="K17" s="75">
+        <v>6</v>
+      </c>
+      <c r="L17" s="118"/>
+      <c r="M17" s="125"/>
+      <c r="N17" s="126"/>
+      <c r="O17" s="124"/>
       <c r="P17" s="1"/>
       <c r="Q17" s="1"/>
       <c r="R17" s="1"/>
@@ -6602,43 +6606,43 @@
       <c r="V17" s="1"/>
       <c r="W17" s="1"/>
     </row>
-    <row r="18" spans="1:23" s="62" customFormat="1" ht="15" x14ac:dyDescent="0.25">
-      <c r="A18" s="69"/>
-      <c r="B18" s="70"/>
-      <c r="C18" s="70">
-        <v>1</v>
-      </c>
-      <c r="D18" s="70">
-        <v>2</v>
-      </c>
-      <c r="E18" s="70">
-        <v>1</v>
-      </c>
-      <c r="F18" s="70">
-        <v>1</v>
-      </c>
-      <c r="G18" s="70">
-        <v>1</v>
-      </c>
-      <c r="H18" s="70">
-        <v>1</v>
-      </c>
-      <c r="I18" s="70">
-        <v>1</v>
-      </c>
-      <c r="J18" s="70">
-        <v>1</v>
-      </c>
-      <c r="K18" s="82">
-        <v>1</v>
-      </c>
-      <c r="L18" s="128">
+    <row r="18" spans="1:23" ht="15" x14ac:dyDescent="0.25">
+      <c r="A18" s="63"/>
+      <c r="B18" s="64"/>
+      <c r="C18" s="64">
+        <v>1</v>
+      </c>
+      <c r="D18" s="64">
+        <v>2</v>
+      </c>
+      <c r="E18" s="64">
+        <v>1</v>
+      </c>
+      <c r="F18" s="64">
+        <v>1</v>
+      </c>
+      <c r="G18" s="64">
+        <v>1</v>
+      </c>
+      <c r="H18" s="64">
+        <v>1</v>
+      </c>
+      <c r="I18" s="64">
+        <v>1</v>
+      </c>
+      <c r="J18" s="64">
+        <v>1</v>
+      </c>
+      <c r="K18" s="76">
+        <v>1</v>
+      </c>
+      <c r="L18" s="118">
         <f>SUM(C18:K18)</f>
         <v>10</v>
       </c>
-      <c r="M18" s="135"/>
-      <c r="N18" s="136"/>
-      <c r="O18" s="134"/>
+      <c r="M18" s="125"/>
+      <c r="N18" s="126"/>
+      <c r="O18" s="124"/>
       <c r="P18" s="1"/>
       <c r="Q18" s="1"/>
       <c r="R18" s="1"/>
@@ -6655,7 +6659,7 @@
         <f>C17-C18</f>
         <v>5</v>
       </c>
-      <c r="D19" s="73">
+      <c r="D19" s="67">
         <f t="shared" ref="D19:K19" si="4">D17-D18</f>
         <v>4</v>
       </c>
@@ -6675,7 +6679,7 @@
         <f t="shared" si="4"/>
         <v>4</v>
       </c>
-      <c r="I19" s="73">
+      <c r="I19" s="67">
         <f t="shared" si="4"/>
         <v>2</v>
       </c>
@@ -6683,18 +6687,18 @@
         <f t="shared" si="4"/>
         <v>4</v>
       </c>
-      <c r="K19" s="83">
+      <c r="K19" s="77">
         <f t="shared" si="4"/>
         <v>5</v>
       </c>
-      <c r="L19" s="128"/>
-      <c r="M19" s="135">
+      <c r="L19" s="118"/>
+      <c r="M19" s="125">
         <v>0.5</v>
       </c>
-      <c r="N19" s="136">
+      <c r="N19" s="126">
         <v>2.2200000000000002</v>
       </c>
-      <c r="O19" s="134">
+      <c r="O19" s="124">
         <v>2</v>
       </c>
       <c r="P19" s="1"/>
@@ -6735,13 +6739,13 @@
       <c r="J20" s="12">
         <v>5</v>
       </c>
-      <c r="K20" s="81">
-        <v>6</v>
-      </c>
-      <c r="L20" s="128"/>
-      <c r="M20" s="135"/>
-      <c r="N20" s="136"/>
-      <c r="O20" s="134"/>
+      <c r="K20" s="75">
+        <v>6</v>
+      </c>
+      <c r="L20" s="118"/>
+      <c r="M20" s="125"/>
+      <c r="N20" s="126"/>
+      <c r="O20" s="124"/>
       <c r="P20" s="1"/>
       <c r="Q20" s="1"/>
       <c r="R20" s="1"/>
@@ -6751,43 +6755,43 @@
       <c r="V20" s="1"/>
       <c r="W20" s="1"/>
     </row>
-    <row r="21" spans="1:23" s="62" customFormat="1" ht="15" x14ac:dyDescent="0.25">
-      <c r="A21" s="69"/>
-      <c r="B21" s="70"/>
-      <c r="C21" s="70">
-        <v>1</v>
-      </c>
-      <c r="D21" s="70">
-        <v>1</v>
-      </c>
-      <c r="E21" s="70">
-        <v>1</v>
-      </c>
-      <c r="F21" s="70">
+    <row r="21" spans="1:23" ht="15" x14ac:dyDescent="0.25">
+      <c r="A21" s="63"/>
+      <c r="B21" s="64"/>
+      <c r="C21" s="64">
+        <v>1</v>
+      </c>
+      <c r="D21" s="64">
+        <v>1</v>
+      </c>
+      <c r="E21" s="64">
+        <v>1</v>
+      </c>
+      <c r="F21" s="64">
         <v>0</v>
       </c>
-      <c r="G21" s="70">
-        <v>1</v>
-      </c>
-      <c r="H21" s="70">
-        <v>1</v>
-      </c>
-      <c r="I21" s="70">
-        <v>1</v>
-      </c>
-      <c r="J21" s="70">
-        <v>1</v>
-      </c>
-      <c r="K21" s="82">
-        <v>1</v>
-      </c>
-      <c r="L21" s="128">
+      <c r="G21" s="64">
+        <v>1</v>
+      </c>
+      <c r="H21" s="64">
+        <v>1</v>
+      </c>
+      <c r="I21" s="64">
+        <v>1</v>
+      </c>
+      <c r="J21" s="64">
+        <v>1</v>
+      </c>
+      <c r="K21" s="76">
+        <v>1</v>
+      </c>
+      <c r="L21" s="118">
         <f>SUM(C21:K21)</f>
         <v>8</v>
       </c>
-      <c r="M21" s="135"/>
-      <c r="N21" s="136"/>
-      <c r="O21" s="134"/>
+      <c r="M21" s="125"/>
+      <c r="N21" s="126"/>
+      <c r="O21" s="124"/>
       <c r="P21" s="1"/>
       <c r="Q21" s="1"/>
       <c r="R21" s="1"/>
@@ -6832,16 +6836,16 @@
         <f t="shared" si="5"/>
         <v>4</v>
       </c>
-      <c r="K22" s="83">
+      <c r="K22" s="77">
         <f t="shared" si="5"/>
         <v>5</v>
       </c>
-      <c r="L22" s="128"/>
-      <c r="M22" s="135">
+      <c r="L22" s="118"/>
+      <c r="M22" s="125">
         <v>0</v>
       </c>
-      <c r="N22" s="136"/>
-      <c r="O22" s="134"/>
+      <c r="N22" s="126"/>
+      <c r="O22" s="124"/>
       <c r="P22" s="1"/>
       <c r="Q22" s="1"/>
       <c r="R22" s="1"/>
@@ -6880,13 +6884,13 @@
       <c r="J23" s="12">
         <v>6</v>
       </c>
-      <c r="K23" s="81">
+      <c r="K23" s="75">
         <v>7</v>
       </c>
-      <c r="L23" s="128"/>
-      <c r="M23" s="135"/>
-      <c r="N23" s="136"/>
-      <c r="O23" s="134"/>
+      <c r="L23" s="118"/>
+      <c r="M23" s="125"/>
+      <c r="N23" s="126"/>
+      <c r="O23" s="124"/>
       <c r="P23" s="1"/>
       <c r="Q23" s="1"/>
       <c r="R23" s="1"/>
@@ -6896,43 +6900,43 @@
       <c r="V23" s="1"/>
       <c r="W23" s="1"/>
     </row>
-    <row r="24" spans="1:23" s="62" customFormat="1" ht="15" x14ac:dyDescent="0.25">
-      <c r="A24" s="69"/>
-      <c r="B24" s="70"/>
-      <c r="C24" s="70">
-        <v>3</v>
-      </c>
-      <c r="D24" s="70">
-        <v>3</v>
-      </c>
-      <c r="E24" s="70">
-        <v>3</v>
-      </c>
-      <c r="F24" s="70">
-        <v>2</v>
-      </c>
-      <c r="G24" s="70">
-        <v>2</v>
-      </c>
-      <c r="H24" s="70">
-        <v>2</v>
-      </c>
-      <c r="I24" s="70">
-        <v>2</v>
-      </c>
-      <c r="J24" s="70">
-        <v>2</v>
-      </c>
-      <c r="K24" s="82">
-        <v>3</v>
-      </c>
-      <c r="L24" s="128">
+    <row r="24" spans="1:23" ht="15" x14ac:dyDescent="0.25">
+      <c r="A24" s="63"/>
+      <c r="B24" s="64"/>
+      <c r="C24" s="64">
+        <v>3</v>
+      </c>
+      <c r="D24" s="64">
+        <v>3</v>
+      </c>
+      <c r="E24" s="64">
+        <v>3</v>
+      </c>
+      <c r="F24" s="64">
+        <v>2</v>
+      </c>
+      <c r="G24" s="64">
+        <v>2</v>
+      </c>
+      <c r="H24" s="64">
+        <v>2</v>
+      </c>
+      <c r="I24" s="64">
+        <v>2</v>
+      </c>
+      <c r="J24" s="64">
+        <v>2</v>
+      </c>
+      <c r="K24" s="76">
+        <v>3</v>
+      </c>
+      <c r="L24" s="118">
         <f>SUM(C24:K24)</f>
         <v>22</v>
       </c>
-      <c r="M24" s="135"/>
-      <c r="N24" s="136"/>
-      <c r="O24" s="134"/>
+      <c r="M24" s="125"/>
+      <c r="N24" s="126"/>
+      <c r="O24" s="124"/>
       <c r="P24" s="1"/>
       <c r="Q24" s="1"/>
       <c r="R24" s="1"/>
@@ -6945,7 +6949,7 @@
     <row r="25" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="15"/>
       <c r="B25" s="16"/>
-      <c r="C25" s="73">
+      <c r="C25" s="67">
         <f>C23-C24</f>
         <v>3</v>
       </c>
@@ -6957,11 +6961,11 @@
         <f t="shared" si="6"/>
         <v>5</v>
       </c>
-      <c r="F25" s="73">
+      <c r="F25" s="67">
         <f t="shared" si="6"/>
         <v>2</v>
       </c>
-      <c r="G25" s="73">
+      <c r="G25" s="67">
         <f t="shared" si="6"/>
         <v>2</v>
       </c>
@@ -6977,18 +6981,18 @@
         <f t="shared" si="6"/>
         <v>4</v>
       </c>
-      <c r="K25" s="83">
+      <c r="K25" s="77">
         <f t="shared" si="6"/>
         <v>4</v>
       </c>
-      <c r="L25" s="128"/>
-      <c r="M25" s="135">
-        <v>2</v>
-      </c>
-      <c r="N25" s="136">
+      <c r="L25" s="118"/>
+      <c r="M25" s="125">
+        <v>2</v>
+      </c>
+      <c r="N25" s="126">
         <v>8.8800000000000008</v>
       </c>
-      <c r="O25" s="134">
+      <c r="O25" s="124">
         <v>9</v>
       </c>
       <c r="P25" s="1"/>
@@ -7029,13 +7033,13 @@
       <c r="J26" s="12">
         <v>6</v>
       </c>
-      <c r="K26" s="81">
-        <v>5</v>
-      </c>
-      <c r="L26" s="128"/>
-      <c r="M26" s="135"/>
-      <c r="N26" s="136"/>
-      <c r="O26" s="134"/>
+      <c r="K26" s="75">
+        <v>5</v>
+      </c>
+      <c r="L26" s="118"/>
+      <c r="M26" s="125"/>
+      <c r="N26" s="126"/>
+      <c r="O26" s="124"/>
       <c r="P26" s="1"/>
       <c r="Q26" s="1"/>
       <c r="R26" s="1"/>
@@ -7045,43 +7049,43 @@
       <c r="V26" s="1"/>
       <c r="W26" s="1"/>
     </row>
-    <row r="27" spans="1:23" s="62" customFormat="1" ht="15" x14ac:dyDescent="0.25">
-      <c r="A27" s="69"/>
-      <c r="B27" s="70"/>
-      <c r="C27" s="70">
-        <v>2</v>
-      </c>
-      <c r="D27" s="70">
-        <v>2</v>
-      </c>
-      <c r="E27" s="70">
-        <v>2</v>
-      </c>
-      <c r="F27" s="70">
-        <v>1</v>
-      </c>
-      <c r="G27" s="70">
-        <v>2</v>
-      </c>
-      <c r="H27" s="70">
-        <v>1</v>
-      </c>
-      <c r="I27" s="70">
-        <v>1</v>
-      </c>
-      <c r="J27" s="70">
-        <v>2</v>
-      </c>
-      <c r="K27" s="82">
-        <v>2</v>
-      </c>
-      <c r="L27" s="128">
+    <row r="27" spans="1:23" ht="15" x14ac:dyDescent="0.25">
+      <c r="A27" s="63"/>
+      <c r="B27" s="64"/>
+      <c r="C27" s="64">
+        <v>2</v>
+      </c>
+      <c r="D27" s="64">
+        <v>2</v>
+      </c>
+      <c r="E27" s="64">
+        <v>2</v>
+      </c>
+      <c r="F27" s="64">
+        <v>1</v>
+      </c>
+      <c r="G27" s="64">
+        <v>2</v>
+      </c>
+      <c r="H27" s="64">
+        <v>1</v>
+      </c>
+      <c r="I27" s="64">
+        <v>1</v>
+      </c>
+      <c r="J27" s="64">
+        <v>2</v>
+      </c>
+      <c r="K27" s="76">
+        <v>2</v>
+      </c>
+      <c r="L27" s="118">
         <f>SUM(C27:K27)</f>
         <v>15</v>
       </c>
-      <c r="M27" s="135"/>
-      <c r="N27" s="136"/>
-      <c r="O27" s="134"/>
+      <c r="M27" s="125"/>
+      <c r="N27" s="126"/>
+      <c r="O27" s="124"/>
       <c r="P27" s="1"/>
       <c r="Q27" s="1"/>
       <c r="R27" s="1"/>
@@ -7130,12 +7134,12 @@
         <f t="shared" si="7"/>
         <v>3</v>
       </c>
-      <c r="L28" s="129"/>
-      <c r="M28" s="137">
+      <c r="L28" s="119"/>
+      <c r="M28" s="127">
         <v>0</v>
       </c>
-      <c r="N28" s="138"/>
-      <c r="O28" s="141"/>
+      <c r="N28" s="128"/>
+      <c r="O28" s="131"/>
       <c r="P28" s="1"/>
       <c r="Q28" s="1"/>
       <c r="R28" s="1"/>
@@ -7146,7 +7150,7 @@
       <c r="W28" s="1"/>
     </row>
     <row r="29" spans="1:23" ht="15" x14ac:dyDescent="0.25">
-      <c r="O29" s="142"/>
+      <c r="O29" s="132"/>
     </row>
     <row r="30" spans="1:23" ht="15" x14ac:dyDescent="0.25">
       <c r="C30" s="62" t="s">
@@ -7176,11 +7180,11 @@
       <c r="K30" s="62" t="s">
         <v>48</v>
       </c>
-      <c r="N30" s="77">
+      <c r="N30" s="71">
         <f>SUM(N7:N29)</f>
         <v>39.96</v>
       </c>
-      <c r="O30" s="143">
+      <c r="O30" s="133">
         <f>SUM(O7:O29)</f>
         <v>39</v>
       </c>
@@ -8344,23 +8348,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="A1" s="63" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" s="64"/>
-      <c r="C1" s="64"/>
-      <c r="D1" s="64"/>
-      <c r="E1" s="64"/>
-      <c r="F1" s="64"/>
-      <c r="G1" s="64"/>
-      <c r="H1" s="64"/>
-      <c r="I1" s="64"/>
-      <c r="J1" s="64"/>
-      <c r="K1" s="64"/>
-      <c r="L1" s="64"/>
-      <c r="M1" s="64"/>
-      <c r="N1" s="64"/>
-      <c r="O1" s="64"/>
+      <c r="A1" s="139" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="140"/>
+      <c r="C1" s="140"/>
+      <c r="D1" s="140"/>
+      <c r="E1" s="140"/>
+      <c r="F1" s="140"/>
+      <c r="G1" s="140"/>
+      <c r="H1" s="140"/>
+      <c r="I1" s="140"/>
+      <c r="J1" s="140"/>
+      <c r="K1" s="140"/>
+      <c r="L1" s="140"/>
+      <c r="M1" s="140"/>
+      <c r="N1" s="140"/>
+      <c r="O1" s="140"/>
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
       <c r="R1" s="1"/>
@@ -8374,23 +8378,23 @@
       <c r="Z1" s="1"/>
     </row>
     <row r="2" spans="1:26" ht="15" x14ac:dyDescent="0.25">
-      <c r="A2" s="65" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="64"/>
-      <c r="C2" s="64"/>
-      <c r="D2" s="64"/>
-      <c r="E2" s="64"/>
-      <c r="F2" s="64"/>
-      <c r="G2" s="64"/>
-      <c r="H2" s="64"/>
-      <c r="I2" s="64"/>
-      <c r="J2" s="64"/>
-      <c r="K2" s="64"/>
-      <c r="L2" s="64"/>
-      <c r="M2" s="64"/>
-      <c r="N2" s="64"/>
-      <c r="O2" s="64"/>
+      <c r="A2" s="141" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="140"/>
+      <c r="C2" s="140"/>
+      <c r="D2" s="140"/>
+      <c r="E2" s="140"/>
+      <c r="F2" s="140"/>
+      <c r="G2" s="140"/>
+      <c r="H2" s="140"/>
+      <c r="I2" s="140"/>
+      <c r="J2" s="140"/>
+      <c r="K2" s="140"/>
+      <c r="L2" s="140"/>
+      <c r="M2" s="140"/>
+      <c r="N2" s="140"/>
+      <c r="O2" s="140"/>
       <c r="P2" s="1"/>
       <c r="Q2" s="1"/>
       <c r="R2" s="1"/>
@@ -9294,23 +9298,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="A1" s="63" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" s="64"/>
-      <c r="C1" s="64"/>
-      <c r="D1" s="64"/>
-      <c r="E1" s="64"/>
-      <c r="F1" s="64"/>
-      <c r="G1" s="64"/>
-      <c r="H1" s="64"/>
-      <c r="I1" s="64"/>
-      <c r="J1" s="64"/>
-      <c r="K1" s="64"/>
-      <c r="L1" s="64"/>
-      <c r="M1" s="64"/>
-      <c r="N1" s="64"/>
-      <c r="O1" s="64"/>
+      <c r="A1" s="139" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="140"/>
+      <c r="C1" s="140"/>
+      <c r="D1" s="140"/>
+      <c r="E1" s="140"/>
+      <c r="F1" s="140"/>
+      <c r="G1" s="140"/>
+      <c r="H1" s="140"/>
+      <c r="I1" s="140"/>
+      <c r="J1" s="140"/>
+      <c r="K1" s="140"/>
+      <c r="L1" s="140"/>
+      <c r="M1" s="140"/>
+      <c r="N1" s="140"/>
+      <c r="O1" s="140"/>
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
       <c r="R1" s="1"/>
@@ -9324,23 +9328,23 @@
       <c r="Z1" s="1"/>
     </row>
     <row r="2" spans="1:26" ht="15" x14ac:dyDescent="0.25">
-      <c r="A2" s="65" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="64"/>
-      <c r="C2" s="64"/>
-      <c r="D2" s="64"/>
-      <c r="E2" s="64"/>
-      <c r="F2" s="64"/>
-      <c r="G2" s="64"/>
-      <c r="H2" s="64"/>
-      <c r="I2" s="64"/>
-      <c r="J2" s="64"/>
-      <c r="K2" s="64"/>
-      <c r="L2" s="64"/>
-      <c r="M2" s="64"/>
-      <c r="N2" s="64"/>
-      <c r="O2" s="64"/>
+      <c r="A2" s="141" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="140"/>
+      <c r="C2" s="140"/>
+      <c r="D2" s="140"/>
+      <c r="E2" s="140"/>
+      <c r="F2" s="140"/>
+      <c r="G2" s="140"/>
+      <c r="H2" s="140"/>
+      <c r="I2" s="140"/>
+      <c r="J2" s="140"/>
+      <c r="K2" s="140"/>
+      <c r="L2" s="140"/>
+      <c r="M2" s="140"/>
+      <c r="N2" s="140"/>
+      <c r="O2" s="140"/>
       <c r="P2" s="1"/>
       <c r="Q2" s="1"/>
       <c r="R2" s="1"/>
@@ -10976,23 +10980,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="A1" s="63" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" s="64"/>
-      <c r="C1" s="64"/>
-      <c r="D1" s="64"/>
-      <c r="E1" s="64"/>
-      <c r="F1" s="64"/>
-      <c r="G1" s="64"/>
-      <c r="H1" s="64"/>
-      <c r="I1" s="64"/>
-      <c r="J1" s="64"/>
-      <c r="K1" s="64"/>
-      <c r="L1" s="64"/>
-      <c r="M1" s="64"/>
-      <c r="N1" s="64"/>
-      <c r="O1" s="64"/>
+      <c r="A1" s="139" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="140"/>
+      <c r="C1" s="140"/>
+      <c r="D1" s="140"/>
+      <c r="E1" s="140"/>
+      <c r="F1" s="140"/>
+      <c r="G1" s="140"/>
+      <c r="H1" s="140"/>
+      <c r="I1" s="140"/>
+      <c r="J1" s="140"/>
+      <c r="K1" s="140"/>
+      <c r="L1" s="140"/>
+      <c r="M1" s="140"/>
+      <c r="N1" s="140"/>
+      <c r="O1" s="140"/>
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
       <c r="R1" s="1"/>
@@ -11006,23 +11010,23 @@
       <c r="Z1" s="1"/>
     </row>
     <row r="2" spans="1:26" ht="15" x14ac:dyDescent="0.25">
-      <c r="A2" s="65" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="64"/>
-      <c r="C2" s="64"/>
-      <c r="D2" s="64"/>
-      <c r="E2" s="64"/>
-      <c r="F2" s="64"/>
-      <c r="G2" s="64"/>
-      <c r="H2" s="64"/>
-      <c r="I2" s="64"/>
-      <c r="J2" s="64"/>
-      <c r="K2" s="64"/>
-      <c r="L2" s="64"/>
-      <c r="M2" s="64"/>
-      <c r="N2" s="64"/>
-      <c r="O2" s="64"/>
+      <c r="A2" s="141" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="140"/>
+      <c r="C2" s="140"/>
+      <c r="D2" s="140"/>
+      <c r="E2" s="140"/>
+      <c r="F2" s="140"/>
+      <c r="G2" s="140"/>
+      <c r="H2" s="140"/>
+      <c r="I2" s="140"/>
+      <c r="J2" s="140"/>
+      <c r="K2" s="140"/>
+      <c r="L2" s="140"/>
+      <c r="M2" s="140"/>
+      <c r="N2" s="140"/>
+      <c r="O2" s="140"/>
       <c r="P2" s="1"/>
       <c r="Q2" s="1"/>
       <c r="R2" s="1"/>
@@ -11926,23 +11930,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="17.25" x14ac:dyDescent="0.4">
-      <c r="A1" s="66" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" s="67"/>
-      <c r="C1" s="67"/>
-      <c r="D1" s="67"/>
-      <c r="E1" s="67"/>
-      <c r="F1" s="67"/>
-      <c r="G1" s="67"/>
-      <c r="H1" s="67"/>
-      <c r="I1" s="67"/>
-      <c r="J1" s="67"/>
-      <c r="K1" s="67"/>
-      <c r="L1" s="67"/>
-      <c r="M1" s="67"/>
-      <c r="N1" s="67"/>
-      <c r="O1" s="67"/>
+      <c r="A1" s="142" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="143"/>
+      <c r="C1" s="143"/>
+      <c r="D1" s="143"/>
+      <c r="E1" s="143"/>
+      <c r="F1" s="143"/>
+      <c r="G1" s="143"/>
+      <c r="H1" s="143"/>
+      <c r="I1" s="143"/>
+      <c r="J1" s="143"/>
+      <c r="K1" s="143"/>
+      <c r="L1" s="143"/>
+      <c r="M1" s="143"/>
+      <c r="N1" s="143"/>
+      <c r="O1" s="143"/>
       <c r="P1" s="38"/>
       <c r="Q1" s="38"/>
       <c r="R1" s="38"/>
@@ -11956,23 +11960,23 @@
       <c r="Z1" s="38"/>
     </row>
     <row r="2" spans="1:26" ht="15" x14ac:dyDescent="0.25">
-      <c r="A2" s="68" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="67"/>
-      <c r="C2" s="67"/>
-      <c r="D2" s="67"/>
-      <c r="E2" s="67"/>
-      <c r="F2" s="67"/>
-      <c r="G2" s="67"/>
-      <c r="H2" s="67"/>
-      <c r="I2" s="67"/>
-      <c r="J2" s="67"/>
-      <c r="K2" s="67"/>
-      <c r="L2" s="67"/>
-      <c r="M2" s="67"/>
-      <c r="N2" s="67"/>
-      <c r="O2" s="67"/>
+      <c r="A2" s="144" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="143"/>
+      <c r="C2" s="143"/>
+      <c r="D2" s="143"/>
+      <c r="E2" s="143"/>
+      <c r="F2" s="143"/>
+      <c r="G2" s="143"/>
+      <c r="H2" s="143"/>
+      <c r="I2" s="143"/>
+      <c r="J2" s="143"/>
+      <c r="K2" s="143"/>
+      <c r="L2" s="143"/>
+      <c r="M2" s="143"/>
+      <c r="N2" s="143"/>
+      <c r="O2" s="143"/>
       <c r="P2" s="38"/>
       <c r="Q2" s="38"/>
       <c r="R2" s="38"/>
@@ -12438,23 +12442,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="A1" s="63" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" s="64"/>
-      <c r="C1" s="64"/>
-      <c r="D1" s="64"/>
-      <c r="E1" s="64"/>
-      <c r="F1" s="64"/>
-      <c r="G1" s="64"/>
-      <c r="H1" s="64"/>
-      <c r="I1" s="64"/>
-      <c r="J1" s="64"/>
-      <c r="K1" s="64"/>
-      <c r="L1" s="64"/>
-      <c r="M1" s="64"/>
-      <c r="N1" s="64"/>
-      <c r="O1" s="64"/>
+      <c r="A1" s="139" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="140"/>
+      <c r="C1" s="140"/>
+      <c r="D1" s="140"/>
+      <c r="E1" s="140"/>
+      <c r="F1" s="140"/>
+      <c r="G1" s="140"/>
+      <c r="H1" s="140"/>
+      <c r="I1" s="140"/>
+      <c r="J1" s="140"/>
+      <c r="K1" s="140"/>
+      <c r="L1" s="140"/>
+      <c r="M1" s="140"/>
+      <c r="N1" s="140"/>
+      <c r="O1" s="140"/>
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
       <c r="R1" s="1"/>
@@ -12468,23 +12472,23 @@
       <c r="Z1" s="1"/>
     </row>
     <row r="2" spans="1:26" ht="15" x14ac:dyDescent="0.25">
-      <c r="A2" s="65" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="64"/>
-      <c r="C2" s="64"/>
-      <c r="D2" s="64"/>
-      <c r="E2" s="64"/>
-      <c r="F2" s="64"/>
-      <c r="G2" s="64"/>
-      <c r="H2" s="64"/>
-      <c r="I2" s="64"/>
-      <c r="J2" s="64"/>
-      <c r="K2" s="64"/>
-      <c r="L2" s="64"/>
-      <c r="M2" s="64"/>
-      <c r="N2" s="64"/>
-      <c r="O2" s="64"/>
+      <c r="A2" s="141" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="140"/>
+      <c r="C2" s="140"/>
+      <c r="D2" s="140"/>
+      <c r="E2" s="140"/>
+      <c r="F2" s="140"/>
+      <c r="G2" s="140"/>
+      <c r="H2" s="140"/>
+      <c r="I2" s="140"/>
+      <c r="J2" s="140"/>
+      <c r="K2" s="140"/>
+      <c r="L2" s="140"/>
+      <c r="M2" s="140"/>
+      <c r="N2" s="140"/>
+      <c r="O2" s="140"/>
       <c r="P2" s="1"/>
       <c r="Q2" s="1"/>
       <c r="R2" s="1"/>
@@ -13494,43 +13498,43 @@
     <col min="2" max="2" width="12.42578125" style="62" customWidth="1"/>
     <col min="3" max="11" width="10.7109375" style="62" customWidth="1"/>
     <col min="12" max="12" width="6.85546875" style="62" customWidth="1"/>
-    <col min="13" max="13" width="6" style="76" customWidth="1"/>
-    <col min="14" max="14" width="7.140625" style="77" customWidth="1"/>
+    <col min="13" max="13" width="6" style="70" customWidth="1"/>
+    <col min="14" max="14" width="7.140625" style="71" customWidth="1"/>
     <col min="15" max="15" width="8.7109375" style="35" customWidth="1"/>
     <col min="16" max="23" width="8.7109375" style="62" customWidth="1"/>
     <col min="24" max="16384" width="14.140625" style="62"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" s="88" customFormat="1" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="84" t="s">
+    <row r="1" spans="1:23" s="80" customFormat="1" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="145" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="85"/>
-      <c r="C1" s="85"/>
-      <c r="D1" s="85"/>
-      <c r="E1" s="85"/>
-      <c r="F1" s="85"/>
-      <c r="G1" s="85"/>
-      <c r="H1" s="85"/>
-      <c r="I1" s="85"/>
-      <c r="J1" s="85"/>
-      <c r="K1" s="85"/>
-      <c r="L1" s="85"/>
-      <c r="M1" s="89" t="s">
+      <c r="B1" s="146"/>
+      <c r="C1" s="146"/>
+      <c r="D1" s="146"/>
+      <c r="E1" s="146"/>
+      <c r="F1" s="146"/>
+      <c r="G1" s="146"/>
+      <c r="H1" s="146"/>
+      <c r="I1" s="146"/>
+      <c r="J1" s="146"/>
+      <c r="K1" s="146"/>
+      <c r="L1" s="146"/>
+      <c r="M1" s="81" t="s">
         <v>54</v>
       </c>
-      <c r="N1" s="86"/>
-      <c r="O1" s="90" t="s">
+      <c r="N1" s="78"/>
+      <c r="O1" s="82" t="s">
         <v>55</v>
       </c>
-      <c r="P1" s="87"/>
-      <c r="Q1" s="87"/>
-      <c r="R1" s="87"/>
-      <c r="S1" s="87"/>
-      <c r="T1" s="87"/>
-      <c r="U1" s="87"/>
-      <c r="V1" s="87"/>
-      <c r="W1" s="87"/>
+      <c r="P1" s="79"/>
+      <c r="Q1" s="79"/>
+      <c r="R1" s="79"/>
+      <c r="S1" s="79"/>
+      <c r="T1" s="79"/>
+      <c r="U1" s="79"/>
+      <c r="V1" s="79"/>
+      <c r="W1" s="79"/>
     </row>
     <row r="2" spans="1:23" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A2" s="19" t="s">
@@ -13566,12 +13570,12 @@
       <c r="K2" s="20">
         <v>9</v>
       </c>
-      <c r="L2" s="78" t="s">
+      <c r="L2" s="72" t="s">
         <v>7</v>
       </c>
-      <c r="M2" s="91"/>
-      <c r="N2" s="95"/>
-      <c r="O2" s="99"/>
+      <c r="M2" s="83"/>
+      <c r="N2" s="87"/>
+      <c r="O2" s="91"/>
       <c r="P2" s="3"/>
       <c r="Q2" s="3"/>
       <c r="R2" s="3"/>
@@ -13613,10 +13617,10 @@
       <c r="K3" s="6">
         <v>5</v>
       </c>
-      <c r="L3" s="79"/>
-      <c r="M3" s="92"/>
-      <c r="N3" s="96"/>
-      <c r="O3" s="100"/>
+      <c r="L3" s="73"/>
+      <c r="M3" s="84"/>
+      <c r="N3" s="88"/>
+      <c r="O3" s="92"/>
       <c r="P3" s="3"/>
       <c r="Q3" s="3"/>
       <c r="R3" s="3"/>
@@ -13658,10 +13662,10 @@
       <c r="K4" s="25">
         <v>2</v>
       </c>
-      <c r="L4" s="80"/>
-      <c r="M4" s="92"/>
-      <c r="N4" s="96"/>
-      <c r="O4" s="100"/>
+      <c r="L4" s="74"/>
+      <c r="M4" s="84"/>
+      <c r="N4" s="88"/>
+      <c r="O4" s="92"/>
       <c r="P4" s="3"/>
       <c r="Q4" s="3"/>
       <c r="R4" s="3"/>
@@ -13705,10 +13709,10 @@
       <c r="K5" s="12">
         <v>8</v>
       </c>
-      <c r="L5" s="81"/>
-      <c r="M5" s="93"/>
-      <c r="N5" s="97"/>
-      <c r="O5" s="100"/>
+      <c r="L5" s="75"/>
+      <c r="M5" s="85"/>
+      <c r="N5" s="89"/>
+      <c r="O5" s="92"/>
       <c r="P5" s="1"/>
       <c r="Q5" s="1"/>
       <c r="R5" s="1"/>
@@ -13719,44 +13723,44 @@
       <c r="W5" s="1"/>
     </row>
     <row r="6" spans="1:23" ht="15" x14ac:dyDescent="0.25">
-      <c r="A6" s="69"/>
-      <c r="B6" s="70" t="s">
+      <c r="A6" s="63"/>
+      <c r="B6" s="64" t="s">
         <v>40</v>
       </c>
-      <c r="C6" s="70">
-        <v>2</v>
-      </c>
-      <c r="D6" s="70">
-        <v>2</v>
-      </c>
-      <c r="E6" s="70">
-        <v>2</v>
-      </c>
-      <c r="F6" s="70">
-        <v>3</v>
-      </c>
-      <c r="G6" s="70">
-        <v>2</v>
-      </c>
-      <c r="H6" s="70">
-        <v>3</v>
-      </c>
-      <c r="I6" s="70">
-        <v>3</v>
-      </c>
-      <c r="J6" s="70">
-        <v>2</v>
-      </c>
-      <c r="K6" s="70">
-        <v>2</v>
-      </c>
-      <c r="L6" s="82">
+      <c r="C6" s="64">
+        <v>2</v>
+      </c>
+      <c r="D6" s="64">
+        <v>2</v>
+      </c>
+      <c r="E6" s="64">
+        <v>2</v>
+      </c>
+      <c r="F6" s="64">
+        <v>3</v>
+      </c>
+      <c r="G6" s="64">
+        <v>2</v>
+      </c>
+      <c r="H6" s="64">
+        <v>3</v>
+      </c>
+      <c r="I6" s="64">
+        <v>3</v>
+      </c>
+      <c r="J6" s="64">
+        <v>2</v>
+      </c>
+      <c r="K6" s="64">
+        <v>2</v>
+      </c>
+      <c r="L6" s="76">
         <f>SUM(C6:K6)</f>
         <v>21</v>
       </c>
-      <c r="M6" s="93"/>
-      <c r="N6" s="97"/>
-      <c r="O6" s="100"/>
+      <c r="M6" s="85"/>
+      <c r="N6" s="89"/>
+      <c r="O6" s="92"/>
       <c r="P6" s="1"/>
       <c r="Q6" s="1"/>
       <c r="R6" s="1"/>
@@ -13771,7 +13775,7 @@
       <c r="B7" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="C7" s="73">
+      <c r="C7" s="67">
         <f>C5-C6</f>
         <v>4</v>
       </c>
@@ -13791,11 +13795,11 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="H7" s="73">
+      <c r="H7" s="67">
         <f t="shared" si="0"/>
         <v>2</v>
       </c>
-      <c r="I7" s="73">
+      <c r="I7" s="67">
         <f t="shared" si="0"/>
         <v>2</v>
       </c>
@@ -13803,18 +13807,18 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="K7" s="73">
+      <c r="K7" s="67">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="L7" s="83"/>
-      <c r="M7" s="93">
-        <v>2</v>
-      </c>
-      <c r="N7" s="97">
+      <c r="L7" s="77"/>
+      <c r="M7" s="85">
+        <v>2</v>
+      </c>
+      <c r="N7" s="89">
         <v>4.4400000000000004</v>
       </c>
-      <c r="O7" s="100">
+      <c r="O7" s="92">
         <v>4</v>
       </c>
       <c r="P7" s="1"/>
@@ -13860,10 +13864,10 @@
       <c r="K8" s="12">
         <v>8</v>
       </c>
-      <c r="L8" s="81"/>
-      <c r="M8" s="93"/>
-      <c r="N8" s="97"/>
-      <c r="O8" s="100"/>
+      <c r="L8" s="75"/>
+      <c r="M8" s="85"/>
+      <c r="N8" s="89"/>
+      <c r="O8" s="92"/>
       <c r="P8" s="1"/>
       <c r="Q8" s="1"/>
       <c r="R8" s="1"/>
@@ -13874,44 +13878,44 @@
       <c r="W8" s="1"/>
     </row>
     <row r="9" spans="1:23" ht="15" x14ac:dyDescent="0.25">
-      <c r="A9" s="69"/>
-      <c r="B9" s="70" t="s">
+      <c r="A9" s="63"/>
+      <c r="B9" s="64" t="s">
         <v>40</v>
       </c>
-      <c r="C9" s="70">
-        <v>2</v>
-      </c>
-      <c r="D9" s="70">
-        <v>2</v>
-      </c>
-      <c r="E9" s="70">
-        <v>2</v>
-      </c>
-      <c r="F9" s="70">
-        <v>1</v>
-      </c>
-      <c r="G9" s="70">
-        <v>2</v>
-      </c>
-      <c r="H9" s="70">
-        <v>2</v>
-      </c>
-      <c r="I9" s="70">
-        <v>2</v>
-      </c>
-      <c r="J9" s="70">
-        <v>2</v>
-      </c>
-      <c r="K9" s="70">
-        <v>2</v>
-      </c>
-      <c r="L9" s="82">
+      <c r="C9" s="64">
+        <v>2</v>
+      </c>
+      <c r="D9" s="64">
+        <v>2</v>
+      </c>
+      <c r="E9" s="64">
+        <v>2</v>
+      </c>
+      <c r="F9" s="64">
+        <v>1</v>
+      </c>
+      <c r="G9" s="64">
+        <v>2</v>
+      </c>
+      <c r="H9" s="64">
+        <v>2</v>
+      </c>
+      <c r="I9" s="64">
+        <v>2</v>
+      </c>
+      <c r="J9" s="64">
+        <v>2</v>
+      </c>
+      <c r="K9" s="64">
+        <v>2</v>
+      </c>
+      <c r="L9" s="76">
         <f>SUM(C9:K9)</f>
         <v>17</v>
       </c>
-      <c r="M9" s="93"/>
-      <c r="N9" s="97"/>
-      <c r="O9" s="100"/>
+      <c r="M9" s="85"/>
+      <c r="N9" s="89"/>
+      <c r="O9" s="92"/>
       <c r="P9" s="1"/>
       <c r="Q9" s="1"/>
       <c r="R9" s="1"/>
@@ -13942,7 +13946,7 @@
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
-      <c r="G10" s="73">
+      <c r="G10" s="67">
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
@@ -13954,22 +13958,22 @@
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
-      <c r="J10" s="73">
+      <c r="J10" s="67">
         <f t="shared" si="1"/>
         <v>2</v>
       </c>
-      <c r="K10" s="73">
+      <c r="K10" s="67">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="L10" s="83"/>
-      <c r="M10" s="93">
-        <v>3</v>
-      </c>
-      <c r="N10" s="97">
+      <c r="L10" s="77"/>
+      <c r="M10" s="85">
+        <v>3</v>
+      </c>
+      <c r="N10" s="89">
         <v>6.66</v>
       </c>
-      <c r="O10" s="100">
+      <c r="O10" s="92">
         <v>7</v>
       </c>
       <c r="P10" s="1"/>
@@ -14015,10 +14019,10 @@
       <c r="K11" s="12">
         <v>8</v>
       </c>
-      <c r="L11" s="81"/>
-      <c r="M11" s="93"/>
-      <c r="N11" s="97"/>
-      <c r="O11" s="100"/>
+      <c r="L11" s="75"/>
+      <c r="M11" s="85"/>
+      <c r="N11" s="89"/>
+      <c r="O11" s="92"/>
       <c r="P11" s="1"/>
       <c r="Q11" s="1"/>
       <c r="R11" s="1"/>
@@ -14029,44 +14033,44 @@
       <c r="W11" s="1"/>
     </row>
     <row r="12" spans="1:23" ht="15" x14ac:dyDescent="0.25">
-      <c r="A12" s="69"/>
-      <c r="B12" s="70" t="s">
+      <c r="A12" s="63"/>
+      <c r="B12" s="64" t="s">
         <v>40</v>
       </c>
-      <c r="C12" s="70">
-        <v>2</v>
-      </c>
-      <c r="D12" s="70">
-        <v>1</v>
-      </c>
-      <c r="E12" s="70">
-        <v>1</v>
-      </c>
-      <c r="F12" s="70">
-        <v>2</v>
-      </c>
-      <c r="G12" s="70">
-        <v>2</v>
-      </c>
-      <c r="H12" s="70">
-        <v>2</v>
-      </c>
-      <c r="I12" s="70">
-        <v>2</v>
-      </c>
-      <c r="J12" s="70">
-        <v>2</v>
-      </c>
-      <c r="K12" s="70">
-        <v>1</v>
-      </c>
-      <c r="L12" s="82">
+      <c r="C12" s="64">
+        <v>2</v>
+      </c>
+      <c r="D12" s="64">
+        <v>1</v>
+      </c>
+      <c r="E12" s="64">
+        <v>1</v>
+      </c>
+      <c r="F12" s="64">
+        <v>2</v>
+      </c>
+      <c r="G12" s="64">
+        <v>2</v>
+      </c>
+      <c r="H12" s="64">
+        <v>2</v>
+      </c>
+      <c r="I12" s="64">
+        <v>2</v>
+      </c>
+      <c r="J12" s="64">
+        <v>2</v>
+      </c>
+      <c r="K12" s="64">
+        <v>1</v>
+      </c>
+      <c r="L12" s="76">
         <f>SUM(C12:K12)</f>
         <v>15</v>
       </c>
-      <c r="M12" s="93"/>
-      <c r="N12" s="97"/>
-      <c r="O12" s="100"/>
+      <c r="M12" s="85"/>
+      <c r="N12" s="89"/>
+      <c r="O12" s="92"/>
       <c r="P12" s="1"/>
       <c r="Q12" s="1"/>
       <c r="R12" s="1"/>
@@ -14085,7 +14089,7 @@
         <f>C11-C12</f>
         <v>6</v>
       </c>
-      <c r="D13" s="73">
+      <c r="D13" s="67">
         <f t="shared" ref="D13:K13" si="2">D11-D12</f>
         <v>5</v>
       </c>
@@ -14093,11 +14097,11 @@
         <f t="shared" si="2"/>
         <v>5</v>
       </c>
-      <c r="F13" s="73">
+      <c r="F13" s="67">
         <f t="shared" si="2"/>
         <v>2</v>
       </c>
-      <c r="G13" s="73">
+      <c r="G13" s="67">
         <f t="shared" si="2"/>
         <v>4</v>
       </c>
@@ -14105,7 +14109,7 @@
         <f t="shared" si="2"/>
         <v>4</v>
       </c>
-      <c r="I13" s="73">
+      <c r="I13" s="67">
         <f t="shared" si="2"/>
         <v>2</v>
       </c>
@@ -14117,14 +14121,14 @@
         <f t="shared" si="2"/>
         <v>7</v>
       </c>
-      <c r="L13" s="83"/>
-      <c r="M13" s="93">
-        <v>2</v>
-      </c>
-      <c r="N13" s="97">
+      <c r="L13" s="77"/>
+      <c r="M13" s="85">
+        <v>2</v>
+      </c>
+      <c r="N13" s="89">
         <v>4.4400000000000004</v>
       </c>
-      <c r="O13" s="100">
+      <c r="O13" s="92">
         <v>4</v>
       </c>
       <c r="P13" s="1"/>
@@ -14170,10 +14174,10 @@
       <c r="K14" s="12">
         <v>8</v>
       </c>
-      <c r="L14" s="81"/>
-      <c r="M14" s="93"/>
-      <c r="N14" s="97"/>
-      <c r="O14" s="100"/>
+      <c r="L14" s="75"/>
+      <c r="M14" s="85"/>
+      <c r="N14" s="89"/>
+      <c r="O14" s="92"/>
       <c r="P14" s="1"/>
       <c r="Q14" s="1"/>
       <c r="R14" s="1"/>
@@ -14184,44 +14188,44 @@
       <c r="W14" s="1"/>
     </row>
     <row r="15" spans="1:23" ht="15" x14ac:dyDescent="0.25">
-      <c r="A15" s="69"/>
-      <c r="B15" s="70" t="s">
+      <c r="A15" s="63"/>
+      <c r="B15" s="64" t="s">
         <v>40</v>
       </c>
-      <c r="C15" s="70">
-        <v>1</v>
-      </c>
-      <c r="D15" s="70">
-        <v>1</v>
-      </c>
-      <c r="E15" s="70">
-        <v>1</v>
-      </c>
-      <c r="F15" s="70">
-        <v>2</v>
-      </c>
-      <c r="G15" s="70">
-        <v>1</v>
-      </c>
-      <c r="H15" s="70">
-        <v>2</v>
-      </c>
-      <c r="I15" s="70">
-        <v>2</v>
-      </c>
-      <c r="J15" s="70">
-        <v>2</v>
-      </c>
-      <c r="K15" s="70">
-        <v>1</v>
-      </c>
-      <c r="L15" s="82">
+      <c r="C15" s="64">
+        <v>1</v>
+      </c>
+      <c r="D15" s="64">
+        <v>1</v>
+      </c>
+      <c r="E15" s="64">
+        <v>1</v>
+      </c>
+      <c r="F15" s="64">
+        <v>2</v>
+      </c>
+      <c r="G15" s="64">
+        <v>1</v>
+      </c>
+      <c r="H15" s="64">
+        <v>2</v>
+      </c>
+      <c r="I15" s="64">
+        <v>2</v>
+      </c>
+      <c r="J15" s="64">
+        <v>2</v>
+      </c>
+      <c r="K15" s="64">
+        <v>1</v>
+      </c>
+      <c r="L15" s="76">
         <f>SUM(C15:K15)</f>
         <v>13</v>
       </c>
-      <c r="M15" s="93"/>
-      <c r="N15" s="97"/>
-      <c r="O15" s="100"/>
+      <c r="M15" s="85"/>
+      <c r="N15" s="89"/>
+      <c r="O15" s="92"/>
       <c r="P15" s="1"/>
       <c r="Q15" s="1"/>
       <c r="R15" s="1"/>
@@ -14236,7 +14240,7 @@
       <c r="B16" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="C16" s="73">
+      <c r="C16" s="67">
         <f>C14-C15</f>
         <v>4</v>
       </c>
@@ -14244,11 +14248,11 @@
         <f t="shared" ref="D16:K16" si="3">D14-D15</f>
         <v>6</v>
       </c>
-      <c r="E16" s="73">
+      <c r="E16" s="67">
         <f t="shared" si="3"/>
         <v>4</v>
       </c>
-      <c r="F16" s="73">
+      <c r="F16" s="67">
         <f t="shared" si="3"/>
         <v>2</v>
       </c>
@@ -14260,7 +14264,7 @@
         <f t="shared" si="3"/>
         <v>4</v>
       </c>
-      <c r="I16" s="73">
+      <c r="I16" s="67">
         <f t="shared" si="3"/>
         <v>2</v>
       </c>
@@ -14272,14 +14276,14 @@
         <f t="shared" si="3"/>
         <v>7</v>
       </c>
-      <c r="L16" s="83"/>
-      <c r="M16" s="94">
-        <v>2</v>
-      </c>
-      <c r="N16" s="98">
+      <c r="L16" s="77"/>
+      <c r="M16" s="86">
+        <v>2</v>
+      </c>
+      <c r="N16" s="90">
         <v>4.4400000000000004</v>
       </c>
-      <c r="O16" s="147">
+      <c r="O16" s="137">
         <v>4</v>
       </c>
       <c r="P16" s="1"/>
@@ -14292,10 +14296,10 @@
       <c r="W16" s="1"/>
     </row>
     <row r="17" spans="3:15" ht="15" x14ac:dyDescent="0.25">
-      <c r="O17" s="148"/>
+      <c r="O17" s="138"/>
     </row>
     <row r="18" spans="3:15" ht="15" x14ac:dyDescent="0.25">
-      <c r="C18" s="74" t="s">
+      <c r="C18" s="68" t="s">
         <v>45</v>
       </c>
       <c r="D18" s="62" t="s">
@@ -14322,14 +14326,14 @@
       <c r="K18" s="62" t="s">
         <v>46</v>
       </c>
-      <c r="O18" s="148"/>
+      <c r="O18" s="138"/>
     </row>
     <row r="19" spans="3:15" ht="15" x14ac:dyDescent="0.25">
-      <c r="C19" s="75" t="s">
+      <c r="C19" s="69" t="s">
         <v>46</v>
       </c>
-      <c r="D19" s="71"/>
-      <c r="E19" s="71"/>
+      <c r="D19" s="65"/>
+      <c r="E19" s="65"/>
       <c r="F19" s="62" t="s">
         <v>45</v>
       </c>
@@ -14339,11 +14343,11 @@
       <c r="K19" s="62" t="s">
         <v>50</v>
       </c>
-      <c r="N19" s="77">
+      <c r="N19" s="71">
         <f>SUM(N7:N18)</f>
         <v>19.980000000000004</v>
       </c>
-      <c r="O19" s="148">
+      <c r="O19" s="138">
         <f>SUM(O7:O18)</f>
         <v>19</v>
       </c>
@@ -14352,7 +14356,7 @@
       <c r="C20" s="29"/>
     </row>
     <row r="21" spans="3:15" x14ac:dyDescent="0.2">
-      <c r="C21" s="72"/>
+      <c r="C21" s="66"/>
     </row>
     <row r="22" spans="3:15" x14ac:dyDescent="0.2">
       <c r="C22" s="29"/>
@@ -14383,23 +14387,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="A1" s="63" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" s="64"/>
-      <c r="C1" s="64"/>
-      <c r="D1" s="64"/>
-      <c r="E1" s="64"/>
-      <c r="F1" s="64"/>
-      <c r="G1" s="64"/>
-      <c r="H1" s="64"/>
-      <c r="I1" s="64"/>
-      <c r="J1" s="64"/>
-      <c r="K1" s="64"/>
-      <c r="L1" s="64"/>
-      <c r="M1" s="64"/>
-      <c r="N1" s="64"/>
-      <c r="O1" s="64"/>
+      <c r="A1" s="139" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="140"/>
+      <c r="C1" s="140"/>
+      <c r="D1" s="140"/>
+      <c r="E1" s="140"/>
+      <c r="F1" s="140"/>
+      <c r="G1" s="140"/>
+      <c r="H1" s="140"/>
+      <c r="I1" s="140"/>
+      <c r="J1" s="140"/>
+      <c r="K1" s="140"/>
+      <c r="L1" s="140"/>
+      <c r="M1" s="140"/>
+      <c r="N1" s="140"/>
+      <c r="O1" s="140"/>
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
       <c r="R1" s="1"/>
@@ -14413,23 +14417,23 @@
       <c r="Z1" s="1"/>
     </row>
     <row r="2" spans="1:26" ht="15" x14ac:dyDescent="0.25">
-      <c r="A2" s="65" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="64"/>
-      <c r="C2" s="64"/>
-      <c r="D2" s="64"/>
-      <c r="E2" s="64"/>
-      <c r="F2" s="64"/>
-      <c r="G2" s="64"/>
-      <c r="H2" s="64"/>
-      <c r="I2" s="64"/>
-      <c r="J2" s="64"/>
-      <c r="K2" s="64"/>
-      <c r="L2" s="64"/>
-      <c r="M2" s="64"/>
-      <c r="N2" s="64"/>
-      <c r="O2" s="64"/>
+      <c r="A2" s="141" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="140"/>
+      <c r="C2" s="140"/>
+      <c r="D2" s="140"/>
+      <c r="E2" s="140"/>
+      <c r="F2" s="140"/>
+      <c r="G2" s="140"/>
+      <c r="H2" s="140"/>
+      <c r="I2" s="140"/>
+      <c r="J2" s="140"/>
+      <c r="K2" s="140"/>
+      <c r="L2" s="140"/>
+      <c r="M2" s="140"/>
+      <c r="N2" s="140"/>
+      <c r="O2" s="140"/>
       <c r="P2" s="1"/>
       <c r="Q2" s="1"/>
       <c r="R2" s="1"/>

</xml_diff>